<commit_message>
fix(ui): refactor decision column and prevent layout flickering
- Implement 'State Lock & Edit' UI in PaperTable.jsx, separating solid Human Decisions from bordered ghost AI Recommendations.
- Fix layout flickering during progress polling by passing an 'isSilent' parameter to fetchPapers, bypassing the full-row loading spinner.
- Resolve calibration papers accumulation bug by strictly resetting 'is_calibration = 0' on all rows before marking a new sample.
- Implement in-memory deduplication prior to drawing the calibration sample in sqlite_repository.py, guaranteeing exactly 100 unique papers are evaluated.
- Fix type-safety for 'source_type' (handling both Enum and String types) during SQLite loading
</commit_message>
<xml_diff>
--- a/data/processed/export/APOLLO_Screening_Results.xlsx
+++ b/data/processed/export/APOLLO_Screening_Results.xlsx
@@ -34,13 +34,13 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00333333"/>
+      <b val="1"/>
+      <color rgb="00C65911"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00C65911"/>
+      <color rgb="00333333"/>
       <sz val="10"/>
     </font>
     <font>
@@ -140,16 +140,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -937,11 +937,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
@@ -974,11 +970,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
@@ -1011,11 +1003,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n"/>
@@ -1048,11 +1036,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
@@ -1130,11 +1114,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
@@ -1167,11 +1147,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
@@ -1204,11 +1180,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
@@ -1286,11 +1258,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
@@ -1368,11 +1336,7 @@
           <t>EC1</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
@@ -1405,11 +1369,7 @@
           <t>EC2; EC5</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
@@ -1442,11 +1402,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
@@ -1479,11 +1435,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
@@ -1516,11 +1468,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
@@ -1598,11 +1546,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="n"/>
@@ -1635,11 +1579,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="n"/>
@@ -1672,11 +1612,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="n"/>
@@ -1709,11 +1645,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
@@ -1746,11 +1678,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="n"/>
@@ -1828,11 +1756,7 @@
           <t>EC4</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
@@ -1865,11 +1789,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="n"/>
@@ -1902,11 +1822,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="n"/>
@@ -1939,11 +1855,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
@@ -1976,11 +1888,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
@@ -2013,11 +1921,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
@@ -2050,11 +1954,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
@@ -2087,11 +1987,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
@@ -2214,11 +2110,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
@@ -2251,11 +2143,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
@@ -2288,11 +2176,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
@@ -2325,11 +2209,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
@@ -2362,11 +2242,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="n"/>
@@ -2489,11 +2365,7 @@
           <t>EC2; EC4</t>
         </is>
       </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
@@ -2526,11 +2398,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="n"/>
@@ -2608,11 +2476,7 @@
           <t>EC2</t>
         </is>
       </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
@@ -2690,11 +2554,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="n"/>
@@ -3050,11 +2910,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I60" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="n"/>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="n"/>
@@ -3095,11 +2951,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I61" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="n"/>
       <c r="K61" s="2" t="n"/>
       <c r="L61" s="2" t="n"/>
@@ -3140,11 +2992,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I62" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="n"/>
       <c r="K62" s="2" t="n"/>
       <c r="L62" s="2" t="n"/>
@@ -3185,11 +3033,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n"/>
       <c r="K63" s="2" t="n"/>
       <c r="L63" s="2" t="n"/>
@@ -3226,11 +3070,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I64" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
@@ -3271,11 +3111,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I65" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="n"/>
@@ -3316,11 +3152,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I66" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
       <c r="L66" s="2" t="n"/>
@@ -3357,9 +3189,9 @@
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="J67" s="2" t="n"/>
@@ -3402,11 +3234,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I68" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="n"/>
       <c r="L68" s="2" t="n"/>
@@ -3447,11 +3275,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="n"/>
       <c r="K69" s="2" t="n"/>
       <c r="L69" s="2" t="n"/>
@@ -3492,11 +3316,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n"/>
       <c r="K70" s="2" t="n"/>
       <c r="L70" s="2" t="n"/>
@@ -3582,11 +3402,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I72" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n"/>
       <c r="K72" s="2" t="n"/>
       <c r="L72" s="2" t="n"/>
@@ -3627,11 +3443,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n"/>
       <c r="K73" s="2" t="n"/>
       <c r="L73" s="2" t="n"/>
@@ -3672,11 +3484,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n"/>
       <c r="K74" s="2" t="n"/>
       <c r="L74" s="2" t="n"/>
@@ -3713,11 +3521,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n"/>
       <c r="K75" s="2" t="n"/>
       <c r="L75" s="2" t="n"/>
@@ -3758,11 +3562,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
       <c r="L76" s="2" t="n"/>
@@ -3803,11 +3603,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="n"/>
       <c r="K77" s="2" t="n"/>
       <c r="L77" s="2" t="n"/>
@@ -3893,9 +3689,9 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="J79" s="2" t="n"/>
@@ -3983,11 +3779,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I81" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="n"/>
       <c r="K81" s="2" t="n"/>
       <c r="L81" s="2" t="n"/>
@@ -4099,9 +3891,7 @@
           <t>Software Engineering Job Market: Salaries, Trends &amp; Insights</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat(ai): implement state-of-the-art Active Learning Cascade (SVM + Few-Shot)
- Introduce dynamic Few-Shot Prompting, injecting human-audited ground truth as memory into Ollama to maximize precision.
- Implement an SVM + TF-IDF fast-track classifier to pre-screen and exclude irrelevant papers in milliseconds on the CPU, bypassing the GPU to drastically reduce full screening time.
</commit_message>
<xml_diff>
--- a/data/processed/export/APOLLO_Screening_Results.xlsx
+++ b/data/processed/export/APOLLO_Screening_Results.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,23 +34,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00C65911"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <color rgb="00333333"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -61,18 +49,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
         <bgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -135,22 +111,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -696,12 +666,12 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -709,30 +679,26 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Big Code Search: A Bibliography</t>
+          <t>Goal-oriented assessment of product-line domains</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Code search is an essential task in software development. Developers often search the internet and other code databases for necessary source code snippets to ease the development efforts. Code search techniques also help learn programming as novice programmers or students can quickly retrieve (hopefully good) examples already used in actual software projects. Given the recurrence of the code search activity in software development, there is an increasing interest in the research community. To improve the code search experience, the research community suggests many code search tools and techniques. These tools and techniques leverage several different ideas and claim a better code search performance. However, it is still challenging to illustrate a comprehensive view of the field considering that existing studies generally explore narrow and limited subsets of used components. This study aims to devise a grounded approach to understanding the procedure for code search and build an operational taxonomy capturing the critical facets of code search techniques. Additionally, we investigate evaluation methods, benchmarks, and datasets used in the field of code search.</t>
+          <t>Software product-line engineering is a method for improving the efficiency and effectiveness of software development. Introducing such a method into an industrial software development environment is potentially of great benefit, but one cannot afford to stop product development while doing so. Rather, in Avaya we apply an incremental adoption strategy and therefore must identify which part(s) of the product line we will create first. Since we consider a product line to consist of a number of domains, the problem is to identify the right domains to start with. We identified two driving factors for selecting product-line domains: corporate impact and likelihood of success. Our assessment of candidate domains is driven by these two goals, which we decompose further into a set of domain selection criteria and corresponding questions. The data, i.e., the answers to the questions, are gathered during interview sessions with our domain experts and evaluated according to our goal decomposition formulas. We illustrate the approach by an example application for which we assessed 20 different domains for one of Avaya's major product lines. © 2003 IEEE.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Code search; code recommendation; code retrieval; find code; code snippet; code search procedure</t>
+          <t>Application programs; Computer architecture; Computer programming; Computer software; Mathematical programming; Product development; Computer industry; Different domains; Domain experts; Driving factors; Goal-oriented; Industrial software development; Selection criteria; Software product line engineerings; Software design</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
@@ -746,7 +712,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1051</t>
+          <t>1006</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -754,30 +720,26 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>How Much Effort Do You Need to Expend on a Technical Interview? A Study of LeetCode Problem Solving Statistics</t>
+          <t>An Exploration of the Perceived Value of Information Technology Certification between Information Technology and Human Resources Professionals</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>A technical interview is the culmination of the recruiting process for hiring software engineers in the tech industry. Many well-known companies, including Amazon, Meta (formerly Facebook), Alphabet (Google), and Microsoft, use it to filter candidates. However, the drawbacks of technical interviews are well-documented, including their lack of real-world relevance, bias towards newer developers, demanding time commitment, and potential to induce unnecessary anxiety and frustration. De-spite these criticisms, there is no clear indication that the industry will alter the format of technical interviews in the near future. To assist student developers in preparing for these challenges, we conducted a quantitative analysis using over 300,000 user profiles from LeetCode, arguably the most popular online platform for preparing software development candidates for interviews. Our analysis aims to provide developers with insights into the effort required to prepare for technical interviews, especially in terms of solving programming questions, to secure a position at a renowned company. © 2024 IEEE.</t>
+          <t>During the decade of the 1990s, many firms engaged in widespread internal dissemination of information technology (IT) in an effort to leverage the capabilities of IT into greater organizational efficiencies. Information technologies such as electronic mail, office automation applications, and enterprise resource planning systems, are a few of the most popular examples of organizational IT initiatives from the past decade. Today, the use of information technology is an integral part of the ordinary course of business and provides technologically progressive firms with heretofore-unseen opportunities. For example, Dell Computers developed and maintains a competitive advantage in the retail technology sector based partly upon the use if information technology that did not exist 10 years ago. Although business applications of information technology present firms with vast opportunity, there is a myriad of complexities associated with organizational IT usage. Generally, this paper examines one critical area: the human resource aspect of organizational IT usage. Specifically, the research presented herein answers the question “Do human resource and information technology professionals perceive information technology certification differently?” The question is of practical relevance when examined, as in this study, within the context of the candidate selection process for a firm evaluating potential hires for an information technology-related position. Initially, the current paper presents a comprehensive overview of the theoretical foundations of certification. From theory, we construct a testing methodology that utilizes, as subjects, practicing human resource and information technology professionals. An analysis of the collected data revealed a marked difference in the perception of information technology certification among the subject groups. Based on the results of structured interviews with the study participants, we present concluding explanations regarding the statistically significant differences among groups. © 2009 by IGI Global. All rights reserved.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Career; Coding challenge; Facebook; Google+; Hiring practices; Leetcode; MicroSoft; Problem-solving; Real-world; Technical interview; Software design</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC4</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>Enterprise resource planning; Information dissemination; Information use; Personnel selection; Automation applications; Enterprise resource planning systems; Information technology certification; Information technology professionals; Information technology usages; Organizational efficiency; Organizational information; Perceived value; Resource professionals; Value of information; Competition</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
@@ -791,7 +753,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1072</t>
+          <t>1017</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -799,26 +761,22 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>“This Gig Is Not for Women”: Gender Stereotyping in Online Hiring</t>
+          <t>Demand and Status of a Scientific Degree in the Non-Academic Labour Market: Regional Case; [Востребованность и статус учёной степени на неакадемическом рынке труда: региональный кейс]</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>This study examines gender segregation in the context of the so-called gig economy. In particular, it explores the role that stereotypes about male and female occupations play in sorting men and women into different jobs in an online freelance marketplace. The findings suggest that gender stereotypes are particularly salient in online hiring because employers typically contract for short-term, relatively low-value jobs based on limited information about job applicants. These conditions trigger the use of cognitive shortcuts about intrinsic gender characteristics linked to different skills and occupations. The results corroborate that female candidates are less likely to be hired for male-typed jobs (e.g., software development) but more likely to be hired for female-typed jobs (e.g., writing and translation) than equally qualified male candidates. Further, the study investigates three mechanisms predicted to attenuate the female penalty in male-typed jobs. The penalty is found to be self-reinforcing, as it perpetuates gender imbalances in worker activity across job categories that strengthen the sex typing of occupations. © The Author(s) 2019.</t>
+          <t>Technological leadership and innovation-driven growth have actualized the request for highly qualified personnel, which have recently been associated with holders of a scientific degree. In the academic field, a scientific degree is a testimony to the occupational status and an integral feature of professional growth and advancement. The reasonableness and significance of a scientific degree in the non-academic market are ambiguous. The purpose of this article is to investigate the opinion and assessments of the non-academic sphere representatives about the demand for the employees with a scientific degree and the status of a scientific degree outside the academic labour market. The research was conducted using the method of semi-structured interview with employers and representatives of seven enterprises in the south of Russia in the machine engineering, metalworking, ferrous metallurgy and IT sectors (n = 13). As a result of the study it was established that: in employment a scientific degree does not give competitive advantages to the applicant; a scientific degree has no value in the non-academic labour market, does not contribute to the advancement and occupation of a higher position in the enterprise; a scientific degree and the presence of employees with a scientific degree in the staff are considered as image-building, status marker and reputation capital of the enterprise; employers have stereotypes regarding scientific employees, which are associated both with the individual organization of labour processes and the compatibility of the scientific, creative and production process; the non-academic sector lacks a human resources strategy for dealing with such employees and a system of their incentives. The authors conclude that the demand for a scientific degree in the non-academic labour market is caused largely by a political request related with the belief that technological and innovative breakthroughs can provide highly qualified personnel with a scientific degree. The authors focus on the probable risks associated with the massification of degree holders, that can lead to a blurring of academic culture and loss of identity of the scientific community. © 2025 Moscow Polytechnic University. All rights reserved.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC3</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>EC1</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
@@ -832,7 +790,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1076</t>
+          <t>1026</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -840,30 +798,22 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Using the DELPHI Method for Model for Role Assignment in the Software Industry</t>
+          <t>Evaluating the effectiveness of E-recruitment in IT companies: Overcoming technological constraints and regulatory compliance</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Over the past two decades, there has been a growing interest in modeling the elements that need to be considered when assigning people to roles in software projects, as evidenced by the number of available publications related to the topic. However, for the most part, these studies, have taken only a partial approach to the issue. Some have focused on the target role's competency profile, while others have tried to understand the preferences of software developers for activities linked to certain roles and the relationship between these preferences and the candidate's personal traits, to mention only two examples. Our research aims to find elements that can be integrated into an allocation model that complements current approaches by including competencies, personal traits, and project team building theories. To do so we performed an expert's consultation exercise using the DELPHI method; which allowed us to validate a set of patterns related to different candidate's personal traits, and the link between the team's motivational motors and their roles within the software development. © 2021 IEEE.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Decision making; Personnel selection; Assigning role in software project; DELPHI method and software engineering; Empirical studies; Personality trait in software project staffing; Personality traits; Software engineering empirical study; Software project; Software project staffing; Software design</t>
-        </is>
-      </c>
+          <t>As the Information Technology industry evolves, e-recruitment emerges as a pivotal tool for sourcing talent. However, challenges like technological constraints and regulatory compliance hinder its effectiveness. This cross-sectional study delves into the discerned effectiveness of e-recruitment methods and the associated barriers encountered by Information Technology companies in the adoption of these practices. A robust dataset comprising responses from 537 participants actively involved in recruitment activities across various sectors of the Information Technology industry was collected through a structured questionnaire. The analysis employed descriptive statistics to summarize sample demographics, inferential statistics including correlation and regression analyses to test hypotheses, and Harman's single-factor test to determine common method variance. The study identified several key findings aligned with its research objectives. Firstly, it confirmed a constructive association between the discerned effectiveness of e-recruitment methods and their adoption by Information Technology companies. However, it also revealed that technological constraints negatively impact the perceived effectiveness of e-recruitment, highlighting a critical barrier in the adoption process. Additionally, the study uncovered a significant association between the availability of skilled Information Technology professionals and the effectiveness of e-recruitment methods utilized by Information Technology firms. Moreover, it found that the integration of e-recruitment platforms with existing human resources systems positively influences their perceived effectiveness in the Information Technology sector, while regulatory compliance requirements pose significant barriers to their effective implementation. Furthermore, the study revealed that the user experience design in e-recruitment platforms affects their perceived effectiveness among Information Technology job seekers and human resources professionals. This study contributes novel insights by providing empirical evidence on the efficacy of e-recruitment methods in Information Technology organizations and the barriers hindering their adoption. Its findings offer insights for Information Technology companies and human resources professionals to enhance their recruitment strategies and address potential challenges, thereby unlocking the potential of e-recruitment in the Information Technology field. © The Author(s) 2025.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>IC1; IC2</t>
+          <t>IC1; IC2; IC3; IC4</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
@@ -877,7 +827,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1095</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -885,26 +835,26 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Analytics for Talent Acquisition: Case of IT Sector in India</t>
+          <t>Assessing technical candidates on the social web</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>One of the challenges faced by Talent Acquisition teams today pertains to the acquisition of human resources by matching job descriptions and skillsets desired. It is more so in the case of competitive sectors like the Indian IT sector. There can be various channels for Talent Acquisition and accordingly, the cost and benefits might vary. However, the consequences of a mismatch have an impact on the quality of deliverables, high recruitment expenses and loss of revenue for the organization. With increased and diverse sources of data that are available to organizations today, there is ample opportunity to apply analytics for informed decision making in this field. This paper reveals useful insights that help streamline the Talent Acquisition process in the Indian IT Industry. The paper adopts a data-centric approach to examine the critical determinants for efficient and effective Talent Acquisition process in IT organizations. Selected supervised machine learning algorithms are applied for the analysis of the dataset. The study is likely to help organizations in reassessing their talent acquisition strategy with respect to key parameters like expected cost to company (CTC), candidate sourcing channels and optimal joining period. © 2020, Asia Pacific Journal of Information Systems. All rights reserved</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC2</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>The Social Web provides comprehensive and publicly available information about software developers, identifying them as contributors to open source projects, experts at maintaining ties on social network sites, or active participants on knowledge-sharing sites. These signals, when aggregated and summarized, could be used to define potential candidates' individual profiles: potential employers could qualitatively evaluate job seekers, even those lacking a formal degree or changing their career path, by assessing candidates' online contributions. At the same time, developers are aware of the Web's public nature and the possible uses of published information when they determine what to share with the world. Some might even try to manipulate public signals of technical qualifications, soft skills, and reputation in their favor. Assessing candidates on the Web for technical positions presents challenges to recruiters, the most serious being the interpretation of the provided signals. An in-depth discussion proposes guidelines for software engineers and recruiters to help recruiters interpret the value and trouble with the signals and metrics they use to assess a candidate's characteristics and skills. © 1984-2012 IEEE.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Computer supported cooperative work; Human computer interaction; Knowledge management; Knowledge representation; Social networking (online); Social sciences computing; Career paths; Group and organization interfaces; Information interfaces; Job seekers; Knowledge retrieval; Knowledge-sharing; Open source projects; Social Networks; Soft skills; Software developer; Software engineers; Technical qualification; Employment</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
@@ -913,12 +863,12 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1145</t>
+          <t>1072</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -926,17 +876,21 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Gender Discrimination in Hiring Decisions: Evidence from a Field Experiment</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+          <t>“This Gig Is Not for Women”: Gender Stereotyping in Online Hiring</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>This study examines gender segregation in the context of the so-called gig economy. In particular, it explores the role that stereotypes about male and female occupations play in sorting men and women into different jobs in an online freelance marketplace. The findings suggest that gender stereotypes are particularly salient in online hiring because employers typically contract for short-term, relatively low-value jobs based on limited information about job applicants. These conditions trigger the use of cognitive shortcuts about intrinsic gender characteristics linked to different skills and occupations. The results corroborate that female candidates are less likely to be hired for male-typed jobs (e.g., software development) but more likely to be hired for female-typed jobs (e.g., writing and translation) than equally qualified male candidates. Further, the study investigates three mechanisms predicted to attenuate the female penalty in male-typed jobs. The penalty is found to be self-reinforcing, as it perpetuates gender imbalances in worker activity across job categories that strengthen the sex typing of occupations. © The Author(s) 2019.</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC3</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
@@ -946,12 +900,12 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1188</t>
+          <t>1084</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -959,15 +913,23 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Unlocking the Value of Artificial Intelligence in Human Resource Management Through Effective Implementation and Usage</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
+          <t>A model for navigating interview processes in requirements elicitation</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Experts in requirements elicitation have interviews to stakeholders using various levels of knowledge to grasp and elicit user's requirements. This paper analyzes interview processes of these experts and explores a computation model for simulating them. This model can be used to navigate novice analysts' interview processes. It is a mixture consisting of a blackboard model and a state transition model in order to narrow the candidates for the questions that an expert analyst will ask the stakeholders next in the interview process. The candidates are selected based on the information that has been elicited from the stakeholders until now, and the blackboard model is for holding this information in the form of IEEE 830, a standard form of requirements specification documents. We have analyzed the experts' interview processes and constructed the instance of the computation model in sales management domain. And we recorded novices' processes, simulated it on the novices' ones, and showed that we could improve them by means of the model.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Computer simulation; Mathematical models; Software engineering; Specifications; Requirements elicitation; Software requirements specification; Requirements engineering</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC4</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -979,12 +941,12 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1195</t>
+          <t>1087</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -992,15 +954,19 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Uncovering the skillsets required in computer science jobs using social network analysis</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
+          <t>Education as a signal of trainability: Results from a vignette study with Italian employers</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Drawing on queuing theory, this study explores the relationship between education and labour market entry from the perspective of employers. On the basis of vignette study, we simulated a hiring process with a sample of recruiters and human resource managers. We analysed the role of education in the screening of applicants' resumes for job openings in the Information, Communication, and Technology sector in the Italian labour market. Findings reveal that employers attach importance to fine-grained indicators of school performance, such as grades and study duration to formulate their hiring decisions, in line with queuing theory. However, internships are disregarded as signals. Results are explained in light of the institutional arrangements that characterize the Italian school-to-work transition system: a standardized education system, poorly specific vocational tracks, weakly developed linkages between schools and firms, a remarkably high dropout rate before study completion. © 2014 © The Author 2014. Published by Oxford University Press. All rights reserved.</t>
+        </is>
+      </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC4</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -1012,12 +978,12 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1199</t>
+          <t>1118</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1025,17 +991,25 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Responsible artificial intelligence in human resources management: a review of the empirical literature</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+          <t>Hiring and Intra-occupational Gender Segregation in Software Engineering</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Women tend to be segregated into different subspecialties than men within male-dominated occupations, but the mechanisms contributing to such intra-occupational gender segregation remain obscure. In this study, I use data from an online recruiting platform and a survey to examine the hiring mechanisms leading to gender segregation within software engineering and development. I find that women are much more prevalent among workers hired in software quality assurance than in other software subspecialties. Importantly, jobs in software quality assurance are lower-paying and perceived as lower status than jobs in other software subspecialties. In examining the origins of this pattern, I find that it stems largely from women being more likely than men to apply for jobs in software quality assurance. Further, such gender differences in job applications are attenuated among candidates with stronger educational credentials, consistent with the idea that relevant accomplishments help mitigate gender differences in self-assessments of competence and belonging in these fields. Demand-side selection processes further contribute to gender segregation, as employers penalize candidates with quality assurance backgrounds, a subspecialty where women are overrepresented, when they apply for jobs in other, higher-status software subspecialties. © American Sociological Association 2020.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>engineering; gender disparity; gender identity; gender relations; labor market; occupation; software; womens employment; womens status; workplace</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC4</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
@@ -1045,12 +1019,12 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>1137</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1058,30 +1032,26 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Cross-national usability study of a housing accessibility app: findings from the European innovage project</t>
+          <t>Automated Question Generation for Technical Interviews Using Deep Learning Models</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>The present usability study concerns an evaluation of an Android based mobile application (app) targeting housing accessibility issues, in a prototype stage for a touch tablet. The objective was to identify and compare elicited usability issues involving senior citizens in two different national contexts: Sweden and Latvia. Applying a problem discovery approach, the study included individual sessions in home environments and follow-up user forums; researchers and user panel participants collaborated to formatively evaluate the app. To support decision-making, the task for the participants was to process information about their present or projected future functional capacity and environmental barriers in their current dwelling. The task was also to make use of a database of professionally assessed available apartments that could be considered for relocation. Data generated in the two countries were analyzed and compared.The results generated new knowledge on relevant usability issues in the two countries and were used to provide design recommendations for the app. The identified usability issues point to a need for a more thorough exploration of design solutions that are tailored for the targeted group of people aging with functional limitations. The results also highlight how national and cultural contexts may influence perceived usability and acceptance and thereby indicate the need to consider these contexts early on and throughout the development process.Tips for usability practitioners: Be aware of possible cross-national differences and handle those challenges in a structured and predefined way, and use real data and real sites to reach close and first-hand experiences.</t>
+          <t>The process of hiring technical talent often demands a thorough and effective evaluation method, though creating interview questions by hand can be slow and lead to uneven results. This paper introduces a tool that automatically generates targeted interview questions from job descriptions, using a specially adjusted BART model. The software, it depends on a selected dataset covering Software Engineering, Cloud Engineering, and Data Science, produces distinct, relevant, and varied questions that are suitable for specific task requirement. Also, it makes use of candidate and recruiter feedback via Reinforcement Learning from Human feedback (RLHF) in order to constantly improve its output, boosting the questions' fit and quality. The experiments using ROUGE metrics show this method not only improves the hiring process but also allows an adaptable way to boost the level of consistency of technical evaluations. © 2025 IEEE.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>ICT products; aging; culture; functional capacity; housing provision; mobile applications; social innovation; software development; user interface; user involvement</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>Deep learning; Employment; Feedback; Job analysis; Software engineering; Automated question generation; BART; Interview question generation; Language processing; Natural language processing; Natural languages; Recruitment automation; Reinforcement learning from human feedback; Reinforcement learnings; Technical interview; Automation</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC2</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
@@ -1090,12 +1060,12 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>1249</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1103,15 +1073,23 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>A Field Study on the Use of Gen AI to Support Computing Education</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
+          <t>Comparative analysis study of open source GIS in Malaysia</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Open source origin might appear like a major prospective change which is qualified to deliver in various industries and also competing means in developing countries. The leading purpose of this research study is to basically discover the degree of adopting Open Source Software (OSS) that is connected with Geographic Information System (GIS) application within Malaysia. It was derived based on inadequate awareness with regards to the origin ideas or even on account of techie deficiencies in the open origin instruments. This particular research has been carried out based on two significant stages; the first stage involved a survey questionnaire: to evaluate the awareness and acceptance level based on the comparison feedback regarding OSS and commercial GIS. This particular survey was conducted among three groups of candidates: government servant, university students and lecturers, as well as individual. The approaches of measuring awareness in this research were based on a comprehending signal plus a notion signal for each survey questions. These kinds of signs had been designed throughout the analysis in order to supply a measurable and also a descriptive signal to produce the final result. The second stage involved an interview session with a major organization that carries out available origin internet GIS; the Federal Department of Town and Country Planning Peninsular Malaysia (JPBD). The impact of this preliminary study was to understand the particular viewpoint of different groups of people on the available origin, and also their insufficient awareness with regards to origin ideas as well as likelihood may be significant root of adopting level connected with available origin options. © Published under licence by IOP Publishing Ltd.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Malaysia; Developing countries; Open source software; Remote sensing; Software engineering; Surveys; Comparative analysis; Federal Department; Internet GIS; Malaysia; Open sources; Open-source GIS; Research studies; University students; comparative study; developing world; GIS; instrumentation; questionnaire survey; software; urban planning; Geographic information systems</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC4</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1123,12 +1101,12 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Scopus</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1286</t>
+          <t>1141</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1136,17 +1114,25 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Start-ups create career opportunities for scientists</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>EC2</t>
-        </is>
-      </c>
+          <t>Searching, examining, and exploiting in-demand technical (SEE IT) skills using web data mining</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>There has always been a mismatch between academic education and industry demands in various industry fields. Especially, in the computer related jobs such as software developers or engineers, employers and job seekers are experiencing a large curriculum or skill gap compared to other industry fields due to its fast-changing nature. In order to minimize the gap, identifying the current job skill trends and offering/learning relevant skills are critically important for both educators and students in the fast-paced job market. However, due to the lack of relative information about the trends of in demand technical skills in certain regions or around the nation, it is difficult for educators to keep up with these changes and determine what needs to be conveyed to students so they can be ready for the job on day one. In this paper, in order to address these challenges, we focused on the analysis of in demand technical skills and their trends in software developer and engineer jobs around the nation. We collected and analyzed over 120,000 software developer or engineer job postings and summarized demanding and required skills from different regions throughout the nation. © 2020 Knowledge Systems Institute Graduate School. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Curricula; Engineers; Software engineering; Students; Academic education; Job postings; Job seekers; Job skills; Relative information; Software developer; Technical skills; Web data mining; Data mining</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>IC1</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
@@ -1161,7 +1147,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1315</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1169,7 +1155,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Comparing Advantages in India’s Computer Hardware and Software Sectors</t>
+          <t>Gender Discrimination in Hiring Decisions: Evidence from a Field Experiment</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
@@ -1189,12 +1175,12 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>1195</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1202,30 +1188,18 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>How Are We Detecting Inconsistent Method Names? An Empirical Study from Code Review Perspective</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Proper naming of methods can make program code easier to understand, and thus enhance software maintainability. Yet, developers may use inconsistent names due to poor communication or a lack of familiarity with conventions within the software development lifecycle. To address this issue, much research effort has been invested into building automatic tools that can check for method name inconsistency and recommend consistent names. However, existing datasets generally do not provide precise details about why a method name was deemed improper and required to be changed. Such information can give useful hints on how to improve the recommendation of adequate method names. Accordingly, we construct a sample method-naming benchmark, ReName4J, by matching name changes with code reviews. We then present an empirical study on how state-of-the-art techniques perform in detecting or recommending consistent and inconsistent method names based on ReName4J. The main purpose of the study is to reveal a different perspective based on reviewed names rather than proposing a complete benchmark. We find that the existing techniques underperform on our review-driven benchmark, both in inconsistent checking and the recommendation. We further identify potential biases in the evaluation of existing techniques, which future research should consider thoroughly.</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Method Name Recommendation; Consistency Checking; Code Review; Empirical Study</t>
-        </is>
-      </c>
+          <t>Uncovering the skillsets required in computer science jobs using social network analysis</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>EC5</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
@@ -1239,7 +1213,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1328</t>
+          <t>1217</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1247,7 +1221,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Success of cloud computing adoption over an era in human resource management systems: a comprehensive meta-analytic literature review</t>
+          <t>AI ethics and governance in business management: challenges, opportunities, and a comparative analysis</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr"/>
@@ -1255,7 +1229,7 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1272,7 +1246,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1280,17 +1254,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ROSE: An IDE-Based Interactive Repair Framework for Debugging</t>
+          <t>Synthesising Privacy by Design Knowledge Toward Explainable Internet of Things Application Designing in Healthcare</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Debugging is costly. Automated program repair (APR) holds the promise of reducing its cost by automatically fixing errors. However, current techniques are not easily applicable in a realistic debugging scenario because they assume a high-quality test suite and frequent program re-execution, have low repair efficiency, and only handle a limited set of errors. To improve the practicality of APR for debugging, we propose ROSE, an interactive repair framework that is able to suggest quick and effective repairs of semantic errors while debugging in an Integrated Development Environment (IDE). ROSE allows an easy integration of existing APR patch generators and can do program repair without assuming the existence of a test suite and without requiring program re-execution. It works in conjunction with an IDE debugger and assumes a debugger stopping point where a problem symptom is observed. ROSE asks the developer to quickly describe the symptom. Then it uses the stopping point, the identified symptom, and the current environment to identify potentially faulty lines, uses a variety of APR techniques to suggest repairs at those lines, and validates those repairs without re-executing the program. Finally, it presents the results so the developer can examine, select, and make the appropriate repair. ROSE uses novel approaches to achieve effective fault localization and patch validation without a test suite or program re-execution. For fault localization, ROSE builds on a fast abstract interpretation-based flow analysis to compute a static backward slice approximating the real dynamic slice while taking into account the symptom and the current execution. For patch validation without re-running the program, ROSE generates simulated traces based on a live-programming system for both the original and repaired executions and compares the traces with respect to the problem symptoms to infer patch correctness. We implemented a prototype of ROSE that works in an Eclipse-based IDE and evaluated its potency and utility with an effectiveness study and a user study. We found that ROSE’s fault localization and validation are highly effective and a ROSE-based tool using existing APR patch generators generated correct repair suggestions for many errors in only seconds. Moreover, the user study demonstrated that ROSE was helpful for debugging and developers liked to use it.</t>
+          <t>Privacy by Design (PbD) is the most common approach followed by software developers who aim to reduce risks within their application designs, yet it remains commonplace for developers to retain little conceptual understanding of what is meant by privacy. A vision is to develop an intelligent privacy assistant to whom developers can easily ask questions to learn how to incorporate different privacy-preserving ideas into their IoT application designs. This article lays the foundations toward developing such a privacy assistant by synthesising existing PbD knowledge to elicit requirements. It is believed that such a privacy assistant should not just prescribe a list of privacy-preserving ideas that developers should incorporate into their design. Instead, it should explain how each prescribed idea helps to protect privacy in a given application design context—this approach is defined as “Explainable Privacy.” A total of 74 privacy patterns were analysed and reviewed using ten different PbD schemes to understand how each privacy pattern is built and how each helps to ensure privacy. Due to page limitations, we have presented a detailed analysis in Reference [3]. In addition, different real-world Internet of Things (IoT) use-cases, including a healthcare application, were used to demonstrate how each privacy pattern could be applied to a given application design. By doing so, several knowledge engineering requirements were identified that need to be considered when developing a privacy assistant. It was also found that, when compared to other IoT application domains, privacy patterns can significantly benefit healthcare applications. In conclusion, this article identifies the research challenges that must be addressed if one wishes to construct an intelligent privacy assistant that can truly augment software developers’ capabilities at the design phase.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Debugging; Interactive Repair Framework; Automated Program Repair; Integrated Development Environment</t>
+          <t>Internet of Things; privacy; privacy by design; privacy assistant; knowledge engineering; healthcare; explainable privacy</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
@@ -1299,11 +1273,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
@@ -1312,12 +1282,12 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>ACM Digital Library</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>128</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1325,15 +1295,23 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Possible Solutions of Wage Problems in Russian IT Market</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
+          <t>A Review of Peer Code Review in Higher Education</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Peer review is the standard process within academia for maintaining publication quality, but it is also widely employed in other settings, such as education and industry, for improving work quality and for generating actionable feedback to content authors. For example, in the software industry peer review of program source code—or peer code review—is a key technique for detecting bugs and maintaining coding standards. In a programming education context, although peer code review offers potential benefits to both code reviewers and code authors, individuals are typically less experienced, which presents a number of challenges. Some of these challenges are similar to those reported in the educational literature on peer review in other academic disciplines, but reviewing code presents unique difficulties. Better understanding these challenges and the conditions under which code review can be taught and implemented successfully in computer science courses is of value to the computing education community. In this work, we conduct a systematic review of the literature on peer code review in higher education to examine instructor motivations for conducting peer code review activities, how such activities have been implemented in practice, and the primary benefits and difficulties that have been reported. We initially identified 187 potential studies and analyzed 51 empirical studies pertinent to our goals. We report the most commonly cited benefits (e.g., the development of programming-related skills) and barriers (e.g., low student engagement), and we identify a wide variety of tools that have been used to facilitate the peer code review process. While we argue that more empirical work is needed to validate currently reported results related to learning outcomes, there is also a clear need to address the challenges around student motivation, which we believe could be an important avenue for future research.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Peer review; code review; higher education; peer code review; programming course; systematic literature review; systematic review</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>EC1</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1345,12 +1323,12 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>ACM Digital Library</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1388</t>
+          <t>129</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1358,15 +1336,23 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Competences for Digital Transformation in Companies – An Analysis of Job Advertisements in Germany</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
+          <t>XCoS: Explainable Code Search Based on Query Scoping and Knowledge Graph</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>When searching code, developers may express additional constraints (e.g., functional constraints and nonfunctional constraints) on the implementations of desired functionalities in the queries. Existing code search tools treat the queries as a whole and ignore the different implications of different parts of the queries. Moreover, these tools usually return a ranked list of candidate code snippets without any explanations. Therefore, the developers often find it hard to choose the desired results and build confidence on them. In this article, we conduct a developer survey to better understand and address these issues and induct some insights from the survey results. Based on the insights, we propose XCoS, an explainable code search approach based on query scoping and knowledge graph. XCoS extracts a background knowledge graph from general knowledge bases like Wikidata and Wikipedia. Given a code search query, XCoS identifies different parts (i.e., functionalities, functional constraints, nonfunctional constraints) from it and use the expressions of functionalities and functional constraints to search the codebase. It then links both the query and the candidate code snippets to the concepts in the background knowledge graph and generates explanations based on the association paths between these two parts of concepts together with relevant descriptions. XCoS uses an interactive user interface that allows the user to better understand the associations between candidate code snippets and the query from different aspects and choose the desired results. Our evaluation shows that the quality of the extracted background knowledge and the concept linkings in codebase is generally high. Furthermore, the generated explanations are considered complete, concise, and readable, and the approach can help developers find the desired code snippets more accurately and confidently.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Code search; explainability; knowledge; concept</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC5</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1383,7 +1369,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>1403</t>
+          <t>1327</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1391,7 +1377,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Challenges and practices of deep learning model reengineering: A case study on computer vision</t>
+          <t>Usage of&amp;#xa0;Generative Artificial Intelligence for&amp;#xa0;the&amp;#xa0;Design of&amp;#xa0;Graphic User Interfaces: Initial Approaches</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr"/>
@@ -1399,7 +1385,7 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1416,7 +1402,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>1408</t>
+          <t>1331</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1424,7 +1410,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Age-related bias and artificial intelligence: a scoping review</t>
+          <t>Achieving a Data-Driven Risk Assessment Methodology for Ethical AI</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
@@ -1432,7 +1418,7 @@
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1444,12 +1430,12 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>ACM Digital Library</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1457,17 +1443,25 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>The Hidden Price of&amp;#xa0;Poor Cooperation – Exploring Industry Perspectives on&amp;#xa0;Social Debt</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+          <t>Impacts of an Industrial Partnership with a Historically Black University on the Computing Career Decisions of Black Undergraduate Students</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>In order to rectify the historical marginalization of Black workers in computing fields, many academic and industrial initiatives have been established to increase the diversity and inclusion in the tech industry. In this study, we explored how one particular post-secondary education program at one historically black institution known as the Google in Residence (GIR) program impacted students’ interests and their pursuit of computing-related careers. Data on employment outcomes at this institution showed that the GIR participants who obtained internships and full-time employment at Google were predominantly international students, not African American students who make up the majority of the undergraduate student and about half of the GIR participants. To understand this phenomenon better, we interviewed 27 students who spanned all 4 years of study and included African American and international students. The interviews were structured to elicit a wide range of factors influencing career decisions. Our analysis describes the impact of a particular GIR introductory-level programming course and other GIR program impacts beyond the introductory-level course. We found that the GIR introductory course was engaging, inspired students to change their degree in a more computing-oriented direction and supported internship applications. The informational workshops, networking events, mock-interviews, and advising of the computer science club, which were supported by the GIR program, built students’ confidence in interviewing and obtaining full-time employment within the tech industry. While the GIR course and program had a positive influence on students of all backgrounds, the reputation of Google was especially motivating for international students. However, the African American students in this study generally had career aspirations and goals that were less tied to specific companies or industries. Based on our findings, potential improvements could include broadening awareness and access of the GIR course to non-computer science majors, offering summer programs to increase students’ computational confidence, and increasing the diversity of GIR and computer science instructors.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>inclusion; internships; industrial partnerships</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC4</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
@@ -1477,12 +1471,12 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>1387</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1490,30 +1484,18 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>ClarifyGPT: A Framework for Enhancing LLM-Based Code Generation via Requirements Clarification</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Large Language Models (LLMs), such as ChatGPT, have demonstrated impressive capabilities in automatically generating code from provided natural language requirements. However, in real-world practice, it is inevitable that the requirements written by users might be ambiguous or insufficient. Current LLMs will directly generate programs according to those unclear requirements, regardless of interactive clarification, which will likely deviate from the original user intents. To bridge that gap, we introduce a novel framework named ClarifyGPT, which aims to enhance code generation by empowering LLMs with the ability to identify ambiguous requirements and ask targeted clarifying questions. Specifically, ClarifyGPT first detects whether a given requirement is ambiguous by performing a code consistency check. If it is ambiguous, ClarifyGPT prompts an LLM to generate targeted clarifying questions. After receiving question responses, ClarifyGPT refines the ambiguous requirement and inputs it into the same LLM to generate a final code solution. To evaluate our ClarifyGPT, we invite ten participants to use ClarifyGPT for code generation on two benchmarks: MBPP-sanitized and MBPP-ET. The results show that ClarifyGPT elevates the performance (Pass@1) of GPT-4 from 70.96% to 80.80% on MBPP-sanitized. Furthermore, to conduct large-scale automated evaluations of ClarifyGPT across different LLMs and benchmarks without requiring user participation, we introduce a high-fidelity simulation method to simulate user responses. The results demonstrate that ClarifyGPT can significantly enhance code generation performance compared to the baselines. In particular, ClarifyGPT improves the average performance of GPT-4 and ChatGPT across five benchmarks from 62.43% to 69.60% and from 54.32% to 62.37%, respectively. A human evaluation also confirms the effectiveness of ClarifyGPT in detecting ambiguous requirements and generating high-quality clarifying questions. We believe that ClarifyGPT can effectively facilitate the practical application of LLMs in real-world development environments.</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Code Generation; Large Language Model; Prompt Engineering</t>
-        </is>
-      </c>
+          <t>Workplace Experiences of Muslim Women in STEM in Canada: An Intersectional Qualitative Analysis</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2; EC4</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n"/>
@@ -1527,7 +1509,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1553</t>
+          <t>1395</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1535,7 +1517,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Jesuit-Informed Casuistry and the Role of Principles for Organizational Ethics</t>
+          <t>Revolutionizing software developmental processes by utilizing continuous software approaches</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
@@ -1543,7 +1525,7 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1560,7 +1542,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1591</t>
+          <t>1518</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1568,7 +1550,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Maximizing Business Potential by Utilizing FinTech Innovative Technologies and Strategies</t>
+          <t>On Using Large Language Models Pre-trained on&amp;#xa0;Digital Twins as&amp;#xa0;Oracles to&amp;#xa0;Foster the&amp;#xa0;Use of&amp;#xa0;Formal Methods in&amp;#xa0;Practice</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
@@ -1576,7 +1558,7 @@
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1593,7 +1575,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>1669</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -1601,7 +1583,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>The Fractional CIO in SMEs: conceptualization and research agenda</t>
+          <t>From Requirements to Prototyping: Proposal and Evaluation of an Artifact to Support Interface Design in the Context of Autism</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr"/>
@@ -1609,7 +1591,7 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1626,7 +1608,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1689</t>
+          <t>1540</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -1634,7 +1616,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Much more than a prediction: Expert-based software effort estimation as a behavioral act</t>
+          <t>Enhancing continuous integration predictions: a hybrid LSTM-GRU deep learning framework with evolved DBSO algorithm</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -1659,7 +1641,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1693</t>
+          <t>1586</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -1667,7 +1649,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>The large language model diagnoses tuberculous pleural effusion in pleural effusion patients through clinical feature landscapes</t>
+          <t>Technology, multidisciplinarianism, and the university</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -1675,7 +1657,7 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1687,12 +1669,12 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>1594</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -1700,30 +1682,18 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Dependency Update Strategies and Package Characteristics</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Managing project dependencies is a key maintenance issue in software development. Developers need to choose an update strategy that allows them to receive important updates and fixes while protecting them from breaking changes. Semantic Versioning was proposed to address this dilemma, but many have opted for more restrictive or permissive alternatives. This empirical study explores the association between package characteristics and the dependency update strategy selected by its dependents to understand how developers select and change their update strategies. We study over 112,000 Node Package Manager (npm) packages and use 19 characteristics to build a prediction model that identifies the common dependency update strategy for each package. Our model achieves a minimum improvement of 72% over the baselines and is much better aligned with community decisions than the npm default strategy. We investigate how different package characteristics can influence the predicted update strategy and find that dependent count, age, and release status to be the highest influencing features. We complement the work with qualitative analyses of 160 packages to investigate the evolution of update strategies. While the common update strategy remains consistent for many packages, certain events such as the release of the 1.0.0 version or breaking changes influence the selected update strategy over time.</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Dependency update strategy; dependency management; software ecosystems; npm</t>
-        </is>
-      </c>
+          <t>An Automated Approach to&amp;#xa0;Identify Source Code Files Affected by&amp;#xa0;Architectural Technical Debt</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="n"/>
@@ -1737,7 +1707,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>1744</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -1745,7 +1715,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Runtime monitoring of operational design domain to safeguard machine learning components</t>
+          <t>Documenting research software in engineering science</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
@@ -1753,7 +1723,7 @@
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1770,7 +1740,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>1746</t>
+          <t>1636</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -1778,7 +1748,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Multimodal Agent AI: A Survey of Recent Advances and Future Directions</t>
+          <t>What is an app store? The software engineering perspective</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
@@ -1803,7 +1773,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1650</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -1811,7 +1781,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Trustworthy AI and Corporate Governance: The EU’s Ethics Guidelines for Trustworthy Artificial Intelligence from a Company Law Perspective</t>
+          <t>Prioritizing unit tests using object-oriented metrics, centrality measures, and machine learning algorithms</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr"/>
@@ -1819,7 +1789,7 @@
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -1836,7 +1806,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1657</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -1844,7 +1814,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>An Integrated Operations and Maintenance Admissions Management System Using Artificial Intelligence Assistance</t>
+          <t>A comprehensive analysis of challenges and strategies for software release notes on GitHub</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
@@ -1852,7 +1822,7 @@
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -1869,7 +1839,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1676</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -1877,7 +1847,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Potential to use metaverse for future teaching and learning</t>
+          <t>A data-driven API recommendation approach for service mashup composition</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1885,7 +1855,7 @@
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC4</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -1902,7 +1872,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>1835</t>
+          <t>1684</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -1910,7 +1880,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Enhancing Research, Learning, and Innovation Through Industry-Academia Synergy with the Industry Interaction Cell Model</t>
+          <t>Enhancing Productivity with&amp;#xa0;AI During the&amp;#xa0;Development of&amp;#xa0;an&amp;#xa0;ISMS: Case Kempower</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
@@ -1918,7 +1888,7 @@
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -1935,7 +1905,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>1849</t>
+          <t>1696</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -1943,7 +1913,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Applying Data Mining Techniques in People Analytics for Balancing Employees’ Interests</t>
+          <t>Potential Candidate Selection Using Information Extraction and Skyline Queries</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr"/>
@@ -1968,7 +1938,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1703</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -1976,7 +1946,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Managing the&amp;#xa0;Root Causes of&amp;#xa0;“Internal API Hell”: An Experience Report</t>
+          <t>Creating of a General Purpose Language for the Construction of Dynamic Reports</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr"/>
@@ -1984,7 +1954,7 @@
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -1996,12 +1966,12 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>1715</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2009,30 +1979,18 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Rust Types for Program Synthesis</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>The Rust type system guarantees memory safety and data-race freedom. However, to satisfy Rust's type rules, many familiar implementation patterns must be adapted substantially. These necessary adaptations complicate programming and might hinder language adoption. In this paper, we demonstrate that, in contrast to manual programming, automatic synthesis is not complicated by Rust's type system, but rather benefits in two major ways. First, a Rust synthesizer can get away with significantly simpler specifications. While in more traditional imperative languages, synthesizers often require lengthy annotations in a complex logic to describe the shape of data structures, aliasing, and potential side effects, in Rust, all this information can be inferred from the types, letting the user focus on specifying functional properties using a slight extension of Rust expressions. Second, the Rust type system reduces the search space for synthesis, which improves performance. In this work, we present the first approach to automatically synthesizing correct-by-construction programs in safe Rust. The key ingredient of our synthesis procedure is Synthetic Ownership Logic, a new program logic for deriving programs that are guaranteed to satisfy both a user-provided functional specification and, importantly, Rust's intricate type system. We implement this logic in a new tool called RusSOL. Our evaluation shows the effectiveness of RusSOL, both in terms of annotation burden and performance, in synthesizing provably correct solutions to common problems faced by new Rust developers.</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Rust; program logic; program synthesis; type systems</t>
-        </is>
-      </c>
+          <t>Method for Eliciting Requirements in the Area of Digital Sovereignty (MERDigS)</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2; EC3</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
@@ -2041,12 +1999,12 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>1719</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2054,30 +2012,18 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Open Collaborative Writing: Investigation of the Fork-and-Pull Model</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Work of all kinds increasingly takes place via networked digital environments that support diverse modes of collaboration. Previous work has investigated how collaborative writing takes place in shared and open workspaces. This study investigates how the "fork-and-pull'' model of distributed version management, now widely utilized in software development, supports coordination and public contribution in collaborative writing. We employ a case study approach to understand coordination around written artifacts in an open pull-based environment. Through interviews and archival analysis of two open text projects: a mathematics textbook on homotopy type theory (HoTT) and open source policies by 18F, a branch of federal agency, we reconstruct how text artifacts were created. We find that in both cases an intensive multi-channel communication among a small core preceded an explicit release action in the form of public communication to solicit broader contribution. Our analysis reveals a dichotomy between two modes of collaboration: a perfecting mode of crafting a public written document versus an evolution mode. In perfecting, authors used the fork-and-pull model to manage contributions refining the text to a more correct version. In evolution, authors used the fork-and-pull model to use a written artifact as a template and starting point, customizing it to their relevant scope. Based on our results, we consider how we might design systems and policies to support pull-based coordination around written artifacts and the forms it takes.</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>case study; coordination; fork-and-pull model; mixed-methods; open collaborative writing; open source model</t>
-        </is>
-      </c>
+          <t>Gender disparity in U.S. patenting</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
@@ -2091,7 +2037,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1729</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2099,7 +2045,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Bridging Business Analysts Competence Gaps: Labor Market Needs Versus Education Standards</t>
+          <t>AI Driving Game Changing Trends in Project Delivery and Enterprise Performance</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2107,7 +2053,7 @@
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2124,7 +2070,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1744</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2132,7 +2078,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Data-driven prototyping via natural-language-based GUI retrieval</t>
+          <t>Runtime monitoring of operational design domain to safeguard machine learning components</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr"/>
@@ -2140,7 +2086,7 @@
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC4</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2157,7 +2103,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>1934</t>
+          <t>1752</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2165,7 +2111,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Mining domain-specific edit operations from model repositories with applications to semantic lifting of model differences and change profiling</t>
+          <t>&lt;span&gt;prompt4vis&lt;/span&gt;: prompting large language models with example mining for tabular data visualization</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2173,7 +2119,7 @@
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2190,7 +2136,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -2198,7 +2144,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Applying a&amp;#xa0;Prompt Pattern Sequence for&amp;#xa0;Decision-Making in&amp;#xa0;Microservices Architectures</t>
+          <t>Operationalising AI governance through ethics-based auditing: an industry case study</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr"/>
@@ -2223,7 +2169,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -2231,7 +2177,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Intermittent control and retinal optic flow when maintaining a curvilinear path</t>
+          <t>Enhancing Research, Learning, and Innovation Through Industry-Academia Synergy with the Industry Interaction Cell Model</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2251,12 +2197,12 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -2264,30 +2210,18 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Inductive Synthesis of Structurally Recursive Functional Programs from Non-recursive Expressions</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>We present a novel approach to synthesizing recursive functional programs from input-output examples. Synthesizing a recursive function is challenging because recursive subexpressions should be constructed while the target function has not been fully defined yet. We address this challenge by using a new technique we call block-based pruning. A block refers to a recursion- and conditional-free expression (i.e., straight-line code) that yields an output from a particular input. We first synthesize as many blocks as possible for each input-output example, and then we explore the space of recursive programs, pruning candidates that are inconsistent with the blocks. Our method is based on an efficient version space learning, thereby effectively dealing with a possibly enormous number of blocks. In addition, we present a method that uses sampled input-output behaviors of library functions to enable a goal-directed search for a recursive program using the library. We have implemented our approach in a system called Trio and evaluated it on synthesis tasks from prior work and on new tasks. Our experiments show that Trio outperforms prior work by synthesizing a solution to 98% of the benchmarks in our benchmark suite.</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Programming by Example; Recursive Functional Programs; Synthesis</t>
-        </is>
-      </c>
+          <t>Data-access performance anti-patterns in data-intensive systems</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
           <t>EC5</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="n"/>
@@ -2296,12 +2230,12 @@
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>1863</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -2309,30 +2243,18 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>"They Can Only Ever Guide": How an Open Source Software Community Uses Roadmaps to Coordinate Effort</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Unlike in commercial software development, open source software (OSS) projects do not generally have managers with direct control over how developers spend their time, yet for projects with large, diverse sets of contributors, the need exists to focus and steer development in a particular direction in a coordinated way. This is especially important for "infrastructure" projects, such as critical libraries and programming languages that many other people depend on. Some projects have taken the approach of borrowing planning tools that originated in commercial development, despite the fact that these techniques were designed for very different contexts, e.g. strong top-down control and profit motives. Little research has been done to understand how these practices are adapted to a new context. In this paper, we examine the Rust project's use of roadmaps: how has an important OSS infrastructure project adapted an inherently top-down tool to the freewheeling world of OSS? We find that because Rust's roadmaps are built in part by summarizing what motivated developers most prefer to work on, they are in some ways more a description of the motivated labor available than they are a directive that the community move in a particular direction. They allow the community to avoid wasting time on unpopular proposals by revealing that there will be little help in building them, and encouraging work on popular features by making visible the amount of consensus in those features. Roadmaps generate a collective focus without limiting the full scope of what developers work on: roadmap issues consume proportionally more effort than other issues, but constitute a minority of the work done (i.e issues and pull requests made) by both central and peripheral participants. They also create transparency among and beyond the community into what central contributors' plans are, and allow more rational decision-making by providing a way for evidence about community needs to be linked to decision-making.</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>collaboration; common pool resources; open source; rust language</t>
-        </is>
-      </c>
+          <t>Configuring Participatory Design of ICT for Aging Well as Matters of Care</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2; EC4</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
@@ -2346,7 +2268,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -2354,7 +2276,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Establishing Effective PhD Supervision for Cross-Disciplinary Research in Advanced Production</t>
+          <t>Revolutionizing User Testing: AI-Powered Feedback with Personalized Personas</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr"/>
@@ -2362,7 +2284,7 @@
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>EC2; EC4</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2379,7 +2301,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2036</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -2387,7 +2309,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>The ethical wisdom of AI developers</t>
+          <t>Competing for Technology Talent: Listed Companies Versus Funded Startups in India</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2407,12 +2329,12 @@
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -2420,30 +2342,18 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Explainable Program Synthesis by Localizing Specifications</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>The traditional formulation of the program synthesis problem is to find a program that meets a logical correctness specification. When synthesis is successful, there is a guarantee that the implementation satisfies the specification. Unfortunately, synthesis engines are typically monolithic algorithms, and obscure the correspondence between the specification, implementation and user intent. In contrast, humans often include comments in their code to guide future developers towards the purpose and design of different parts of the codebase. In this paper, we introduce subspecifications as a mechanism to augment the synthesized implementation with explanatory notes of this form. In this model, the user may ask for explanations of different parts of the implementation; the subspecification generated in response is a logical formula that describes the constraints induced on that subexpression by the global specification and surrounding implementation. We develop algorithms to construct and verify subspecifications and investigate their theoretical properties. We perform an experimental evaluation of the subspecification generation procedure, and measure its effectiveness and running time. Finally, we conduct a user study to determine whether subspecifications are useful: we find that subspecifications greatly aid in understanding the global specification, in identifying alternative implementations, and in debugging faulty implementations.</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Program synthesis; explainability; program comprehension</t>
-        </is>
-      </c>
+          <t>A meta-analysis on social exchange relationships and employee innovation in teams</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
@@ -2457,7 +2367,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2105</t>
+          <t>1958</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -2465,7 +2375,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Towards ensemble-based use case point prediction</t>
+          <t>Modelling the quantification of requirements technical debt</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr"/>
@@ -2473,7 +2383,7 @@
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>EC2</t>
+          <t>EC5</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2490,7 +2400,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>197</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -2498,17 +2408,17 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Automatic Rule Checking for Microservices: Supporting Security Analysis with Explainability</t>
+          <t>Inductive Synthesis of Structurally Recursive Functional Programs from Non-recursive Expressions</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Software security analysis is often done manually, raising performance and correctness issues. Introducing automation is challenging because human verification of the outcomes is often required, especially for security assessment and certification. The distributed nature of microservice applications further increases these concerns.We present an approach for automatically checking architectural security rules on models of microservice applications. It provides explainability for verdicts of rules that are expressed as model queries in our rule specification language. This comprehensible, step-by-step evidence leverages traceability information from the input models to link to artifacts in code. Hence, the complete analysis process from source code via model to rule verdict can be traced and verified. Custom rules can be formulated in addition to a library of 25 best-practice architectural security rules.We evaluated the approach’s correctness by checking the 25 rules on 16 dataflow diagrams of microservice applications with a prototype (called MicroCertiSec) and observed promising results (precision=0.98; recall=1). Additionally, we performed an evaluation with industry experts and academics to gain initial insights into the approach’s usefulness for real-world security analysis. The nine participants gave highly positive feedback on usefulness and usability and stated they would use such an approach in their daily work.</t>
+          <t>We present a novel approach to synthesizing recursive functional programs from input-output examples. Synthesizing a recursive function is challenging because recursive subexpressions should be constructed while the target function has not been fully defined yet. We address this challenge by using a new technique we call block-based pruning. A block refers to a recursion- and conditional-free expression (i.e., straight-line code) that yields an output from a particular input. We first synthesize as many blocks as possible for each input-output example, and then we explore the space of recursive programs, pruning candidates that are inconsistent with the blocks. Our method is based on an efficient version space learning, thereby effectively dealing with a possibly enormous number of blocks. In addition, we present a method that uses sampled input-output behaviors of library functions to enable a goal-directed search for a recursive program using the library. We have implemented our approach in a system called Trio and evaluated it on synthesis tasks from prior work and on new tasks. Our experiments show that Trio outperforms prior work by synthesizing a solution to 98% of the benchmarks in our benchmark suite.</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Security; microservices; software architecture; model-driven engineering; application analysis; dataflow diagrams</t>
+          <t>Programming by Example; Recursive Functional Programs; Synthesis</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
@@ -2517,11 +2427,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="n"/>
@@ -2535,7 +2441,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2119</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -2543,7 +2449,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Towards fair graph-based machine learning software: unveiling and mitigating graph model bias</t>
+          <t>Dynamic Retrieval Augmented Generation of Ontologies using Artificial Intelligence (DRAGON-AI)</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr"/>
@@ -2551,7 +2457,7 @@
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
+          <t>EC2</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -2563,12 +2469,12 @@
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -2576,30 +2482,18 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Understanding the OSS Communities of Deep Learning Frameworks: A Comparative Case Study of PyTorch and TensorFlow</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Over the past two decades, deep learning has received tremendous success in developing software systems across various domains. Deep learning frameworks have been proposed to facilitate the development of such software systems, among which, PyTorch and TensorFlow stand out as notable examples. Considerable attention focuses on exploring software engineering practices and addressing diverse technical aspects in developing and deploying deep learning frameworks and software systems. Despite these efforts, little is known about the open source software communities involved in the development of deep learning frameworks.In this article, we perform a comparative investigation into the open source software communities of the two representative deep learning frameworks, PyTorch and TensorFlow. To facilitate the investigation, we compile a dataset of 2,792 and 3,288 code commit authors, along with 9,826 and 19,750 participants engaged in issue events on GitHub, from the two communities, respectively. With the dataset, we first characterize the structures of the two communities by employing four operationalizations to classify contributors into various roles and inspect the contributions made by common contributors across the two communities. We then conduct a longitudinal analysis to characterize the evolution of the two communities across various releases, in terms of the numbers of contributors with various roles and role transitions among contributors. Finally, we explore the causal effects between community characteristics and the popularity of the two frameworks.We find that the TensorFlow community harbors a larger base of contributors, encompassing a higher proportion of core developers and a more extensive cohort of active users compared to the PyTorch community. In terms of the technical background of the developers, 64.4% and 56.1% developers in the PyTorch and TensorFlow communities are employed by the leading companies of the corresponding open source software projects, Meta and Google, respectively; 25.9% and 21.9% core developers in the PyTorch and TensorFlow communities possess Ph.D. degrees, while 77.2% and 77.7% contribute to other machine learning or deep learning open source projects, respectively. Developers contributing to both communities demonstrate spatial and temporal similarities to some extent in their pull requests across the respective projects. The evolution of contributors with various roles exhibits a consistent upward trend over time in the PyTorch community. Conversely, a noticeable turning point in the growth of contributors characterizes the evolution of the TensorFlow community. Both communities show a statistically significant decreasing trend in the inflow rates of core developers. Furthermore, we observe statistically significant causal effects between the expansion of communities and retention of core developers and the popularity of deep learning frameworks. Based on our findings, we discuss implications, provide recommendations for sustaining open source software communities of deep learning frameworks, and outline directions for future research.</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Deep learning; community evolution; GitHub; developer classification</t>
-        </is>
-      </c>
+          <t>Iran Obesity and Metabolic Surgery (IOMS) Cohort Study: Rationale and Design</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I53" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC2</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="n"/>
@@ -2608,12 +2502,12 @@
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Web of Science</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2207</t>
+          <t>2032</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -2621,30 +2515,18 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Open Source Resume (OSR): A Visualization Tool for Presenting OSS Biographies of Developers</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>In order to recruit appropriate developers for software projects, it is important to have a clarified understanding on the practical experience and expertise of each candidate. However, traditional resume only shows experiences claimed by developers, and very few evidence or information regarding their actual development activities can be obtained. In this paper, we propose an approach to extract developers' practical activities from their participated open source software (OSS) projects, and generate the biographies that reflect their OSS contributions. We applied the approach on the largest code hosting service, GitHub. By investigating the resumes generated from the extracted dataset, recruiters of software projects can be given a clearer view on whether the developers' experiences fulfill the qualifications. Moreover, based on the approach, we present a web-based visualization tool, named as Open Source Resume (OSR). We believe our tool is useful to help recruiters from software development organizations to search for suitable developers, and then construct development teams in software projects based on their OSS contributions.</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>Open Source Software; Mining Software Repositories; Developer Expertise; Visualization Tool</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>IC1</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>Towards fair machine learning using combinatorial methods</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="n"/>
@@ -2653,12 +2535,12 @@
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Web of Science</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2215</t>
+          <t>2103</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -2666,30 +2548,18 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Who is attracted and why? How agile project management influences employee's attraction and commitment</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Purpose In times of market volatility and uncertainty, finding effective strategies to attract and retain individuals continues to be a challenge for organizations. Based on the psychological empowerment process (Spreitzer, 1996), this paper strives to examine if the application of agile project management could serve as such a strategy. Design/methodology/approach In two independent studies, the authors used an experiment with students as potential applicants (N = 121) and a field study with employees (N = 229) to test the predictive quality of agile project management for attracting individuals toward the organization. Findings Using structural equation modeling, the authors identified an indirect relationship between agile project management and attraction toward the organization via psychological empowerment. The authors found this relationship for potential applicants as well as employees. Furthermore, individuals high in sensation seeking are found to be more attracted toward organizations that apply agile project management than individuals low in sensation seeking. Research limitations/implications The findings contribute to the empowerment literature by establishing agile project management as a work structure that fosters feelings of psychological empowerment. Practical implications Taken together, these results suggest that agile project management can attract individuals who seek novel, complex and intense sensations. Where applicable, organizations may highlight their practice of agile project management methodologies as part of their employer brand to attract future specialists for agile projects. Originality/value This paper is the first to integrate the research streams on agile project management and attraction toward the organization using quantitative data.</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>Agile project management; Psychological empowerment; Organizational attractiveness; Organizational commitment; Sensation seeking; Employer branding</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC4</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr"/>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>The Personalized Learning Interaction Framework in Practice (PLIFs): Current Implementations According to Chief Learning Officers and Learning Leaders</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>EC2</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n"/>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="n"/>
@@ -2698,12 +2568,12 @@
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>2126</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -2711,30 +2581,18 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Managing the Transition to Online Freelance Platforms: Self-Directed Socialization</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Individuals increasingly turn to online freelance platforms to find flexible, remote, knowledge-based work. Yet we have only begun to understand the challenges new freelancers face with limited formal resources to orient themselves to this career. To inform design and policy to support new freelancers, we conducted a qualitative interview study on transitions to online freelance platforms with 27 freelancers working on the Upwork and Fiverr platforms. We found that new freelancers engage in self-directed socialization as they proactively seek support not directly provided by the platform or their clients. This support helps them resolve professional identity ambiguity, learn platform work self-management, build credibility, and overcome self-doubt in their new careers. Our findings suggest opportunities to support new forms of socialization and mentorship to address disparities in access to networks, resources, and knowledge needed to successfully begin an online freelance career.</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>career development; future of work; gig economy; mentorship; online freelance platforms; online freelancing; socialization</t>
-        </is>
-      </c>
+          <t>Gamification in software engineering: the mediating role of developer engagement and job satisfaction</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
           <t>EC5</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="n"/>
@@ -2743,12 +2601,12 @@
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>2140</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -2756,30 +2614,18 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>CSM: A Code Style Model for Computing Educators</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Objectives Code style is an important aspect of text-based programming because programs written with good style are considered easier to understand and change and so improve the maintainability of the delivered software product. However teaching code style is complicated by the existence of many style guides and standards that contain inconsistent, low-level advice. The objective of the study is to support educators in helping students understand the nature of these inconsistencies by highlighting the rationale behind rules and their contextual nature.Participants Seventy members of local and national computing science education (CSE) groups contributed in the exploratory phase. Fifty-two members of the ACM SIGCSE members mailing list and the Australasian Chapter contributed in the evaluation and refinement phases. These mailing lists represent a large, global population of CSE educators.Study Methods We created, evaluated and refined an abstract code style model (CSM) comprising a Definition and eight Principles for code style. For CSM creation, we took an exploratory approach based on an examination of the existing literature on code quality and style. To evaluate the level of community endorsement for the model, we analysed quantitative and qualitative data from an international survey questionnaire. We refined the CSM based on an analysis of the qualitative survey data.Findings Analysis of the data from the survey indicated a strong level of support for the CSM. Quantitative data revealed a general agreement with the Principles, with responses for five Principles achieving a minimum of 84 percent agreement and all Principles achieving a minimum of 66 percent agreement. Qualitative data contained very few comments that voiced dissatisfaction with a basic aspect of the model. We found that barriers to developing a community-wide CSM were the strongly-held beliefs about style held by some and the abstract nature of the CSM.Conclusions The creation of an abstract set of Principles for code style is generally perceived by the community to be worthwhile and important and our approach has high levels of endorsement. A validated version of the CSM has been created.</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>computing education; text-based programming; software quality; code style; online survey</t>
-        </is>
-      </c>
+          <t>Distribution-free Bayesian analyses with the DFBA statistical package</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="n"/>
@@ -2788,12 +2634,12 @@
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Web of Science</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>2174</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -2801,30 +2647,26 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Automatically Identifying the Quality of Developer Chats for Post Hoc Use</t>
+          <t>The Evaluation of Founder Failure and Success by Hiring Firms: A Field Experiment</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Software engineers are crowdsourcing answers to their everyday challenges on Q&amp;amp;A forums (e.g., Stack Overflow) and more recently in public chat communities such as Slack, IRC, and Gitter. Many software-related chat conversations contain valuable expert knowledge that is useful for both mining to improve programming support tools and for readers who did not participate in the original chat conversations. However, most chat platforms and communities do not contain built-in quality indicators (e.g., accepted answers, vote counts). Therefore, it is difficult to identify conversations that contain useful information for mining or reading, i.e., conversations of post hoc quality. In this article, we investigate automatically detecting developer conversations of post hoc quality from public chat channels. We first describe an analysis of 400 developer conversations that indicate potential characteristics of post hoc quality, followed by a machine learning-based approach for automatically identifying conversations of post hoc quality. Our evaluation of 2,000 annotated Slack conversations in four programming communities (python, clojure, elm, and racket) indicates that our approach can achieve precision of 0.82, recall of 0.90, F-measure of 0.86, and MCC of 0.57. To our knowledge, this is the first automated technique for detecting developer conversations of post hoc quality.</t>
+          <t>Organizations tout the importance of innovation and entrepreneurship. Yet, when hiring it remains unclear how they evaluate entrepreneurial human capital-namely, job candidates with founder experience. How hiring firms evaluate this experience-and especially how this evaluation varies by entrepreneurial success and failure-reveals insights into the structures and processes within organizations. Organizations research points to two perspectives related to the evaluation of founder experience: Former founders may be advantaged, due to founder experience signaling high-quality capabilities and human capital, or disadvantaged, due to concerns related to fit and commitment. To identify the dominant class of mechanisms driving the evaluation of founder experience, it is important to consider how these evaluations differ, depending on whether the founder's venture failed or succeeded. To isolate demand-side mechanisms and hold supply-side factors constant, we conducted a field experiment. We sent applications varying the candidate's founder experience to 2,400 software engineering positions in the United States at random. We find that former founders received 43% fewer callbacks than nonfounders and that this difference is driven by older hiring firms. Further, this founder penalty is greatest for former successful founders, who received 33% fewer callbacks than former failed founders. Our results highlight that mechanisms related to concerns about fit and commitment, rather than information asymmetry about quality, are most influential when hiring firms evaluate former founders in our context.</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Online software developer chats; quality of social content</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>careers; entrepreneurship; evaluations; failure; experiment; founders; hiring; labor markets</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC2; IC3; IC4; IC5</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="n"/>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="n"/>
@@ -2833,12 +2675,12 @@
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ACM Digital Library</t>
+          <t>Web of Science</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>2214</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -2846,30 +2688,26 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>"A Blocklist is a Boundary": Tensions between Community Protection and Mutual Aid on Federated Social Networks</t>
+          <t>ACHIEVING JOB PERFORMANCE FROM EMPOWERMENT THROUGH THE MEDIATION OF EMPLOYEE ENGAGEMENT: AN EMPIRICAL STUDY</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>The Fediverse (the network encompassing Mastodon, Pleroma, Lemmy, etc.) provides a decentralized alternative to traditional social media platforms, making it both an important refuge for marginalized users and a platform which is well-suited for conducting mutual aid. One emergent type of moderation action for maintaining mutual aid spaces on the Fediverse is the use of community boundary blocklists, which we define as shared lists of Fediverse servers intended to be imported as a common blocklist. However, the use of community boundary blocklists has incited conflict on the Fediverse, with many users left cut off from their communities and sources of support due to actions outside of their control. Using an approach rooted in constructivist grounded theory, we interviewed nine Fediverse users, including a mix of community boundary blocklist curators, server staff, and regular users, to determine key tensions between community moderation and mutual aid practices. From our interviews, we identify the novel perspective of community stewardship as an act of mutual aid. We extend existing collective action and mutual aid frameworks to understand why this perspective conflicts with more typical mutual aid activities. We also observe how federation as a protocol encodes a negative form of consent, allowing users to interact by default and individuals to consent for their entire instance, leading to consent violations. From these insights, we develop a series of community-sourced suggestions for Fediverse platform designers, blocklist curators, and community staff to help address these conflicts and protect marginalized users.</t>
+          <t>In present scenario, business organization understood the importance of sophisticated employee behavior for the development of overall job performance. It is important for an organization to perform effectively for that it enhances their employee's job performance. Many study supports that an empowered employee recognizes and attaches himself or herself with the wider extent of organizational objectives. An engaged employee has more ownership and able to contribute towards his/her own growth and overall productivity. Boston focuses on implementing feedback given by employees with immediate effect and has 43% employees who are highly engaged. Facebook has a culture of contribution and each employee is recognized for his contribution to the overall goal of the company "to make the world more open and connected ". This policy of contributing culture is communicated to all the candidates during recruitment process. That is why Facebook is not only known for being one of the most popular social networking platforms but for its highly engaging culture as well. Under this study, the focus is to understand the relationship between employee empowerment and job performance. The study also tries to explore empirically the mediating effect of employee engagement in this regard. It was conducted on IT sector in Delhi NCR region with a sample size of 182 employees. The finding of the study reflects that engagement has its mediation effect on job performance with respect to employee empowerment.</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>acm proceedings; blocklists; federated networks; fediverse; mastodon; mutual aid; online communities</t>
+          <t>Employee engagement; Employee empowerment; Job Performance; Mediation; Regression</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>EC4</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC5</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="n"/>
@@ -2883,7 +2721,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>231</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -2891,17 +2729,17 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Decision Support Model for Selecting the Optimal Blockchain Oracle Platform: An Evaluation of Key Factors</t>
+          <t>Transformative and Troublesome? Students' and Professional Programmers' Perspectives on Difficult Concepts in Programming</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Smart contract-based applications are executed in a blockchain environment, and they cannot directly access data from external systems, which is required for the service provision of these applications. Instead, smart contracts use agents known as blockchain oracles to collect and provide data feeds to the contracts. The functionality and compatibility with smart contract applications need to be considered when selecting the best-fit oracle platform. As the number of oracle alternatives and their features increases, the decision-making process becomes increasingly complex. Selecting the wrong or sub-optimal oracle is costly and may lead to severe security risks. This article provides a decision support model for the oracle selection problem. The model supports smart contract decision-makers in selecting a secure, cost-effective, and feasible oracle platform for their applications. We interviewed oracle co-founders and smart contracts experts to refine and validate the decision model. Two real-world smart contract application case studies were used to evaluate the model. Our model prioritises and suggests more than one possible oracle platform based on the developer’s required criteria, security assessment and cost analysis. Moreover, this guided decision model serves to reveal issues that may go unnoticed if done haphazardly, reduce decision-making efforts and provide a cost-effective solution.</t>
+          <t>Programming skills are an increasingly desirable asset across disciplines; however, learning to program continues to be difficult for many students. To improve pedagogy, we need to better understand the concepts that students find difficult and which have the biggest impact on their learning. Threshold-concept theory provides a potential lens on student learning, focusing on concepts that are troublesome and transformative. However, there is still a lack of consensus as to what the most relevant threshold concepts in programming are. The challenges involved are related to concept granularity and to evidencing some of the properties expected of threshold concepts. In this article, we report on a qualitative study aiming to address some of these concerns. The study involved focus groups with undergraduate students of different-year groups as well as professional software developers so as to gain insights into how perspectives on concepts change over time. Four concepts emerged from the data, where the majority of participants agreed on their troublesome nature—including abstract classes and data structures. Some of these concepts are considered transformative, too, but the evidence base is weaker. However, even though these concepts may not be considered transformative in the “big” sense of threshold concept theory, we argue the “soft” transformative effect of such concepts means they can provide important guidance for pedagogy and the design of programming courses. Further analysis of the data identified additional concepts that may hinder rather than help the learning of these threshold concepts, which we have called “accidental complexities.” We conclude the article with a critique of the use of threshold concepts as a lens for studying students’ learning of programming.</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>blockchain oracle; smart contracts; technical debt; MCDM</t>
+          <t>Threshold concepts; accidental complexities; computer science curriculum; focus groups; learning programming</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
@@ -2924,7 +2762,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>246</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -2932,17 +2770,17 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>An Empirical Study on the Suitability of Test-based Patch Acceptance Criteria</t>
+          <t>Can GPT-4 Replicate Empirical Software Engineering Research?</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>In this article, we empirically study the suitability of tests as acceptance criteria for automated program fixes, by checking patches produced by automated repair tools using a bug-finding tool, as opposed to previous works that used tests or manual inspections. We develop a number of experiments in which faulty programs from IntroClass, a known benchmark for program repair techniques, are fed to the program repair tools GenProg, Angelix, AutoFix, and Nopol, using test suites of varying quality, including those accompanying the benchmark. We then check the produced patches against formal specifications using a bug-finding tool. Our results show that, in the studied scenarios, automated program repair tools are significantly more likely to accept a spurious program fix than producing an actual one. Using bounded-exhaustive suites larger than the originally given ones (with about 100 and 1,000 tests) we verify that overfitting is reduced but (a) few new correct repairs are generated and (b) some tools see their performance reduced by the larger suites and fewer correct repairs are produced. Finally, by comparing with previous work, we show that overfitting is underestimated in semantics-based tools and that patches not discarded using held-out tests may be discarded using a bug-finding tool.</t>
+          <t>Empirical software engineering research on production systems has brought forth a better understanding of the software engineering process for practitioners and researchers alike. However, only a small subset of production systems is studied, limiting the impact of this research. While software engineering practitioners could benefit from replicating research on their own data, this poses its own set of challenges, since performing replications requires a deep understanding of research methodologies and subtle nuances in software engineering data. Given that large language models (LLMs), such as GPT-4, show promise in tackling both software engineering- and science-related tasks, these models could help replicate and thus democratize empirical software engineering research.In this paper, we examine GPT-4’s abilities to perform replications of empirical software engineering research on new data. We specifically study their ability to surface assumptions made in empirical software engineering research methodologies, as well as their ability to plan and generate code for analysis pipelines on seven empirical software engineering papers. We perform a user study with 14 participants with software engineering research expertise, who evaluate GPT-4-generated assumptions and analysis plans (i.e., a list of module specifications) from the papers. We find that GPT-4 is able to surface correct assumptions, but struggles to generate ones that apply common knowledge about software engineering data. In a manual analysis of the generated code, we find that the GPT-4-generated code contains correct high-level logic, given a subset of the methodology. However, the code contains many small implementation-level errors, reflecting a lack of software engineering knowledge. Our findings have implications for leveraging LLMs for software engineering research as well as practitioner data scientists in software teams.</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>automatic program repair; formal specifications; testing; oracle</t>
+          <t>Large language models; study replication; empirical software engineering</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr"/>
@@ -2965,7 +2803,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>286</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -2973,17 +2811,17 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Cat and Mouse Game: Patching Bureaucratic Work Relations by Patching Technologies</t>
+          <t>Towards Automated Accessibility Report Generation for Mobile Apps</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>This article uses findings from a field study of the world's largest guaranteed employment scheme (NREGA) in India to understand how digital technology mediates work relations and power dynamics within a bureaucracy. In this initiative, upper-level bureaucrats in the south Indian state of Andhra Pradesh built a digital network to remove local discretion at the "last mile" of an implementation of NREGA. I show how digital infrastructure affords actors at both the first and last mile opportunities to modify software to control as well as subvert certain practices. This article refers to this dialectic phenomenon as "governance by patching" and defines it as a socio-technical instantiation of a top-down process that focuses on small changes, iterative, and political process for positive change. Governance by patching is, therefore, neither a purely technical process nor an exclusively administrative one. Rather, it refers to the ability to fix unanticipated problems that arise in the implementation of governance programs by altering the socio-technical systems. The struggle for power continues, but on the new digital terrain.</t>
+          <t>Many apps have basic accessibility issues, like missing labels or low contrast. To supplement manual testing, automated tools can help developers and QA testers find basic accessibility issues, but they can be laborious to use or require writing dedicated tests. To motivate our work, we interviewed eight accessibility QA professionals at a large technology company. From these interviews, we synthesized three design goals for accessibility report generation systems. Motivated by these goals, we developed a system to generate whole app accessibility reports by combining varied data collection methods (e.g., app crawling, manual recording) with an existing accessibility scanner. Many such scanners are based on single-screen scanning, and a key problem in whole app accessibility reporting is to effectively de-duplicate and summarize issues collected across an app. To this end, we developed a screen grouping model with 96.9% accuracy (88.8% F1-score) and UI element matching heuristics with 97% accuracy (98.2% F1-score). We combine these technologies in a system to report and summarize unique issues across an app, and enable a unique pixel-based ignore feature to help engineers and testers better manage reported issues across their app’s lifetime. We conducted a user study where 19 accessibility engineers and testers used multiple tools to create lists of prioritized issues in the context of an accessibility audit. Our system helped them create lists they were more satisfied with while addressing key limitations of current accessibility scanning tools.</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>bureaucracy; governance; ictd; infrastructures; last-mile; nrega; patching</t>
+          <t>UI understanding; app crawling; accessibility</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
@@ -3006,7 +2844,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>293</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -3014,17 +2852,17 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>DesignManager: An Agent-Powered Copilot for Designers to Integrate AI Design Tools into Creative Workflows</t>
+          <t>"Innovative Technologies or Invasive Technologies?": Exploring Design Challenges of Privacy Protection With Smart Home in Jordan</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Creative design is an inherently complex and iterative process characterized by continuous exploration, evaluation, and refinement. While recent advances in generative AI have demonstrated remarkable potential in supporting specific design tasks, there remains a critical gap in understanding how these technologies can enhance the holistic design process rather than just isolated stages. This paper introduces DesignManager, a novel AI-powered design support system that aims to transform how designers collaborate with AI throughout their creative workflow. Through a formative study examining designers' current practices with generative AI, we identified key challenges and opportunities in integrating AI into the creative design process. Based on these insights, we developed DesignManager as an interactive copilot system that provides node-based visualization of design evolution, enabling designers to track, modify, and branch their design processes while maintaining meaningful dialogue-based collaboration. The system offers two collaboration modes: DesignManager-guiding and Designer-guiding. Designers can engage in conversational interactions with the DesignManager to obtain design inspiration and tool recommendations, and proactively advance the design progress. The system employs an agent framework to manage decoupled contextual information emerged during the design process, facilitating deep understanding of designers' needs and providing context-aware assistance. Our technical evaluation validated the effectiveness of context decoupling and the use of agent framework, while the open-ended user study with experts demonstrated that DesignManager successfully supports intuitive intention expression, flexible process control, and deeper creative articulation. This work contributes to the understanding of how AI can evolve from task-specific tools to collaborative partners in creative design processes.</t>
+          <t>The growing adoption of smart devices has fuelled privacy concerns, and prior research has highlighted the privacy of bystanders: individuals who are subjected to the smart device use of others. Most of this research has focused on households in Western contexts (i.e., Europe and North America), but few studies have explored the design challenges of protecting bystanders, and even fewer have explored these in Muslim Arab Middle Eastern settings, such as Jordan.We conduct 44 interviews with users (i.e., families, domestic workers), local and international business leaders, and smart device designers to explore design challenges for privacy protection in the Jordanian context. Our analysis highlights the importance of considering contextual influences and power dynamics, localization and design guidelines, innovative technologies, awareness to design, and regulation. This paper concludes with recommendations for technical, social, business, and legal interventions to improve data protection design of smart devices in Jordan.</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>design copilot; agent; designer-AI collaboration; creative design</t>
+          <t>bystander; design; jordan; privacy; protection; security; smart device; smart home</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
@@ -3047,7 +2885,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>457</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -3055,15 +2893,19 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>HLB: Toward Load-Aware Load Balancing</t>
+          <t>On the Role of Structural Holes in Requirements Identification: An Exploratory Study on Open-Source Software Development</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>The purpose of network load balancers is to optimize quality of service to the users of a set of servers– basically, to improve response times and to reducing computing resources– by properly distributing workloads. This paper proposes a distributed, application-agnostic, Hybrid Load Balancer (HLB) that– without explicit monitoring or signaling– infers server occupancies and processing speeds, which allows making optimised workload placement decisions. This approach is evaluated both through simulations and extensive experiments, including synthetic workloads and Wikipedia replays on a real-world testbed. Results show significant performance gains, in terms of both response time and system utilisation, when compared to existing load-balancing algorithms.</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr"/>
+          <t>Requirements identification is a human-centric activity that involves interaction among multiple stakeholders. Traditional requirements engineering (RE) techniques addressing stakeholders’ social interaction are mainly part of a centralized process intertwined with a specific phase of software development. However, in open-source software (OSS) development, stakeholders’ social interactions are often decentralized, iterative, and dynamic. Little is known about new requirements identification in OSS and the stakeholders’ organizational arrangements supporting such an activity. In this article, we investigate the theory of structural hole from the context of contributing new requirements in OSS projects. Structural hole theory suggests that stakeholders positioned in the structural holes in their social network are able to produce new ideas. In this study, we find that structural hole positions emerge in stakeholders’ social network and these positions are positively related to contributing a higher number of new requirements. We find that along with structural hole positions, stakeholders’ role is also an important part in identifying new requirements. We further observe that structural hole positions evolve over time, thereby identifying requirements to realize enriched features. Our work advances the fundamental understanding of the RE process in a decentralized environment and opens avenues for improved techniques supporting this process.</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Requirements identification; brokerage; open-source requirements engineering; social capital; social information foraging theory; stakeholders’ social network; structural hole</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3084,7 +2926,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>328</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -3092,17 +2934,17 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>A Scoping Review of Informed Consent Practices in Human–Computer Interaction Research</t>
+          <t>An Empirical Study of Self-Admitted Technical Debt in Machine Learning Software</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Obtaining informed consent is a fundamental ethical requirement in research involving human subjects, designed to ensure autonomy, respect, and the protection of participants. However, new technologies and research methodologies in Human–Computer Interaction (HCI) present unique challenges in maintaining ethical standards and require a deeper understanding of how consent practices are implemented. This scoping review provides a detailed examination of the frameworks, methodologies, and practices for obtaining informed consent in HCI. We present recognized universal principles while also discussing the ethical guidelines, and legal frameworks that underpin consent processes. Furthermore, we analyze the practices of disclosure, screening, consenting, and confirmation to assess how researchers ensure voluntary participation. The review addresses key criticisms and challenges identified in the literature, suggesting improvements and exploring alternative approaches. By offering comprehensive insights into the complexities of informed consent, we underscore the ongoing need for ethical awareness and continuous refinement of ethical conduct in HCI.</t>
+          <t>The emergence of open-source ML libraries such as TensorFlow and Google Auto ML has enabled developers to harness state-of-the-art ML algorithms with minimal overhead. However, during this accelerated ML development process, said developers may often make sub-optimal design and implementation decisions, leading to the introduction of technical debt that, if not addressed promptly, can significantly impact on the quality of ML-based software. Developers frequently acknowledge these sub-optimal design and development choices through code comments written during development. These comments, which often highlight areas requiring additional work or refinement in the future are known as self-admitted technical debt (SATD). While prior research has demonstrated that SATD can serve as a reliable indicator of technical debt and has extensively studied SATD in traditional (non-ML) software, little attention has been given to this issue in the context of ML. This paper aims to investigate the occurrence of SATD in ML code by analyzing 318 open-source ML projects across five domains, along with 318 non-ML projects. We detected SATD in source code comments in various snapshots of the studied projects, conducted a manual analysis of a sample of the identified SATD to comprehend the nature of technical debt in the ML code, and performed a survival analysis of the SATD to understand the evolution dynamics of such debts. Our analyses yielded the following observations: (i) Machine learning projects have a median percentage of SATD that is twice that of non-machine learning projects. (ii) ML pipeline stages for data preprocessing and model generation logic are more susceptible to debt than model validation and deployment stages. (iii) SATDs appear in ML projects earlier in the development process compared to non-ML projects. (iv) Long-lasting SATDs are typically introduced during extensive code changes that span multiple files, which exhibit low complexity.Our research contributes to the understanding of technical debt in an ML context and underscores the need for targeted debt management strategies. This contribution is particularly relevant for developers and stakeholders in ML projects by aiding them in identifying and addressing technical debt proactively and paving the way for future research in developing automated tools and methodologies for managing SATD in an ML environment.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Ethical research; informed consent; consent process; consent forms; literature review</t>
+          <t>Self-Admitted Technical Debt; Machine Learning; Survival Analysis; Mining Software Repositories; ML Pipeline; Empirical Software Engineering</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -3125,7 +2967,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>465</t>
+          <t>413</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -3133,17 +2975,17 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>COSTELLO: Contrastive Testing for Embedding-Based Large Language Model as a Service Embeddings</t>
+          <t>A Survey of AIOps in the Era of Large Language Models</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Large language models have gained significant popularity and are often provided as a service (i.e., LLMaaS). Companies like OpenAI and Google provide online APIs of LLMs to allow downstream users to create innovative applications. Despite its popularity, LLM safety and quality assurance is a well-recognized concern in the real world, requiring extra efforts for testing these LLMs. Unfortunately, while end-to-end services like ChatGPT have garnered rising attention in terms of testing, the LLMaaS embeddings have comparatively received less scrutiny. We state the importance of testing and uncovering problematic individual embeddings without considering downstream applications. The abstraction and non-interpretability of embedded vectors, combined with the black-box inaccessibility of LLMaaS, make testing a challenging puzzle. This paper proposes Costello, a black-box approach to reveal potential defects in abstract embedding vectors from LLMaaS by contrastive testing. Our intuition is that high-quality LLMs can adequately capture the semantic relationships of the input texts and properly represent their relationships in the high-dimensional space. For the given interface of LLMaaS and seed inputs, Costello can automatically generate test suites and output words with potential problematic embeddings. The idea is to synthesize contrastive samples with guidance, including positive and negative samples, by mutating seed inputs. Our synthesis guide will leverage task-specific properties to control the mutation procedure and generate samples with known partial relationships in the high-dimensional space. Thus, we can compare the expected relationship (oracle) and embedding distance (output of LLMs) to locate potential buggy cases. We evaluate Costello on 42 open-source (encoder-based) language models and two real-world commercial LLMaaS. Experimental results show that Costello can effectively detect semantic violations, where more than 62% of violations on average result in erroneous behaviors (e.g., unfairness) of downstream applications.</t>
+          <t>As large language models (LLMs) grow increasingly sophisticated and pervasive, their application to various Artificial Intelligence for IT Operations (AIOps) tasks has garnered significant attention. However, a comprehensive understanding of the impact, potential, and limitations of LLMs in AIOps remains in its infancy. To address this gap, we conducted a detailed survey of LLM4AIOps, focusing on how LLMs can optimize processes and improve outcomes in this domain. We analyzed 183 research articles published between January 2020 and December 2024 to answer four key research questions (RQs). In RQ1, we examine the diverse failure data sources utilized, including advanced LLM-based processing techniques for legacy data and the incorporation of new data sources enabled by LLMs. RQ2 explores the evolution of AIOps tasks, highlighting the emergence of novel tasks and the publication trends across these tasks. RQ3 investigates the various LLM-based methods applied to address AIOps challenges. Finally, RQ4 reviews evaluation methodologies tailored to assess LLM-integrated AIOps approaches. Based on our findings, we discuss the state-of-the-art advancements and trends, identify gaps in existing research, and propose promising directions for future exploration.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Software and its engineering → Software testing and debugging; Contrastive Testing; LLMaaS; Embeddings</t>
+          <t>Large language model; AIOps; metrics; logs; time series; incident report; failure perception; anomaly detection; root cause analysis; assisted remediation</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
@@ -3166,7 +3008,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>490</t>
+          <t>468</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -3174,26 +3016,26 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Social Sourcing: Incorporating Social Networks Into Crowdsourcing Contest Design</t>
+          <t>A Stack-Propagation Framework for Low-Resource Personalized Dialogue Generation</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>In a crowdsourcing contest, a principal holding a task posts it to a crowd. People in the crowd then compete with each other to win the rewards. Although in real life, a crowd is usually networked and people influence each other via social ties, existing crowdsourcing contest theories do not aim to answer how interpersonal relationships influence people’s incentives and behaviors and thereby affect the crowdsourcing performance. In this work, we novelly take people’s social ties as a key factor in the modeling and designing of agents’ incentives in crowdsourcing contests. We establish two contest mechanisms by which the principal can impel the agents to invite their neighbors to contribute to the task. The first mechanism has a symmetric Bayesian Nash equilibrium, and it is very simple for agents to play and easy for the principal to predict the contest performance. The second mechanism has an asymmetric Bayesian Nash equilibrium, and agents’ behaviors in equilibrium show a vast diversity which is strongly related to their social relations. The Bayesian Nash equilibrium analysis of these new mechanisms reveals that, besides agents’ intrinsic abilities, the social relations among them also play a central role in decision-making. Moreover, we design an effective algorithm to automatically compute the Bayesian Nash equilibrium of the invitation crowdsourcing contest and further adapt it to a large graph dataset. Both theoretical and empirical results show that the new invitation crowdsourcing contests can substantially enlarge the number of participants, whereby the principal can obtain significantly better solutions without a large advertisement expenditure.</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>IC2; IC4</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>With the resurgent interest in building open-domain dialogue systems, the dialogue generation task has attracted increasing attention over the past few years. This task is usually formulated as a conditional generation problem, which aims to generate a natural and meaningful response given dialogue contexts and specific constraints, such as persona. And maintaining a consistent persona is essential for the dialogue systems to gain trust from the users. Although tremendous advancements have been brought, traditional persona-based dialogue models are typically trained by leveraging a large number of persona-dense dialogue examples. Yet, such persona-dense training data are expensive to obtain, leading to a limited scale. This work presents a novel approach to learning from limited training examples by regarding consistency understanding as a regularization of response generation. To this end, we propose a novel stack-propagation framework for learning a generation and understanding pipeline. Specifically, the framework stacks a Transformer encoder and two Transformer decoders, where the first decoder models response generation and the second serves as a regularizer and jointly models response generation and consistency understanding. The proposed framework can benefit from the stacked encoder and decoders to learn from much smaller personalized dialogue data while maintaining competitive performance. Under different low-resource settings, subjective and objective evaluations prove that the stack-propagation framework outperforms strong baselines in response quality and persona consistency and largely overcomes the shortcomings of traditional models that rely heavily on the persona-dense dialogue data.</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Open-domain dialogue; personalized dialogue generation; stack-propagation; low-resource</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
       <c r="L67" s="2" t="n"/>
@@ -3207,7 +3049,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>477</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -3215,17 +3057,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Fixing Faults in C and Java Source Code: Abbreviated vs. Full-Word Identifier Names</t>
+          <t>Psychometrics in Behavioral Software Engineering: A Methodological Introduction with Guidelines</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>We carried out a family of controlled experiments to investigate whether the use of abbreviated identifier names, with respect to full-word identifier names, affects fault fixing in C and Java source code. This family consists of an original (or baseline) controlled experiment and three replications. We involved 100 participants with different backgrounds and experiences in total. Overall results suggested that there is no difference in terms of effort, effectiveness, and efficiency to fix faults, when source code contains either only abbreviated or only full-word identifier names. We also conducted a qualitative study to understand the values, beliefs, and assumptions that inform and shape fault fixing when identifier names are either abbreviated or full-word. We involved in this qualitative study six professional developers with 1--3 years of work experience. A number of insights emerged from this qualitative study and can be considered a useful complement to the quantitative results from our family of experiments. One of the most interesting insights is that developers, when working on source code with abbreviated identifier names, adopt a more methodical approach to identify and fix faults by extending their focus point and only in a few cases do they expand abbreviated identifiers.</t>
+          <t>A meaningful and deep understanding of the human aspects of software engineering (SE) requires psychological constructs to be considered. Psychology theory can facilitate the systematic and sound development as well as the adoption of instruments (e.g., psychological tests, questionnaires) to assess these constructs. In particular, to ensure high quality, the psychometric properties of instruments need evaluation. In this article, we provide an introduction to psychometric theory for the evaluation of measurement instruments for SE researchers. We present guidelines that enable using existing instruments and developing new ones adequately. We conducted a comprehensive review of the psychology literature framed by the Standards for Educational and Psychological Testing. We detail activities used when operationalizing new psychological constructs, such as item pooling, item review, pilot testing, item analysis, factor analysis, statistical property of items, reliability, validity, and fairness in testing and test bias. We provide an openly available example of a psychometric evaluation based on our guideline. We hope to encourage a culture change in SE research towards the adoption of established methods from psychology. To improve the quality of behavioral research in SE, studies focusing on introducing, validating, and then using psychometric instruments need to be more common.</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>source code identifiers; software testing; replications; qualitative investigation; maintenance; family of experiments; ethnography study; Controlled experiments</t>
+          <t>Empirical software engineering; psychology; behavioral software engineering; methodology; questionnaire design</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
@@ -3248,7 +3090,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -3256,17 +3098,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>An In-Depth Analysis of Occasional and Recurring Collaborations in Online Music Co-creation</t>
+          <t>Market-aware Long-term Job Skill Recommendation with Explainable Deep Reinforcement Learning</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>The success of online creative communities depends on the will of participants to create and derive content in a collaborative environment. Despite their growing popularity, the factors that lead to remixing existing content in online creative communities are not entirely understood. In this article, we focus on overdubbing, a dyadic collaboration in which one author mixes one new track with an audio recording previously uploaded by another. We study musicians who collaborate regularly, frequently overdubbing each other's songs. Building on frequent pattern–mining techniques, we develop an approach to seek instances of such recurring collaborations in the Songtree community. We identify 43 instances involving two or three members with a similar reputation in the community. Our findings highlight common and different remix factors in occasional and recurring collaborations. Specifically, fresh and less mature songs are generally overdubbed more. Exchanging messages and invitations to collaborate are significant factors only for songs generated through recurring collaborations, whereas author reputation (ranking) and applying metadata tags to songs have a positive effect only in occasional collaborations.</t>
+          <t>Continuously learning new skills is essential for talents to gain a competitive advantage in the labor market. Despite extensive efforts on relevance- or preference-based skill recommendations, little attention has been given to the practical effects of job skills in the market. To bridge this gap, we propose an explainable personalized skill learning recommendation system that considers the long-term learning benefits and costs. Specifically, we model skill learning utilities based on salary and learning cost associated with job positions and propose a multi-objective deep reinforcement learning framework to model and maximize long-term utilities. Furthermore, we propose a Self-explaining Skill Recommendation Deep Q-network (SeSRDQN) that captures and prototypes prevalent skill sets in the market into representative exemplars for decision-making. SeSRDQN quantitatively decomposes the talent’s long-term learning utility into contributions from each exemplar, offering a comprehensive and multi-factorial explanation across various skill learning options. To tackle the combinatorial complexity of the skill space, we develop an MCTS-based optimization-decoding iterative training procedure for explanation fidelity and human understandability. In this way, talents will receive a tailored roadmap of essential skills, complemented by exemplar-based explanations, to effectively plan their careers. Extensive experiments on a real-world dataset validate the effectiveness and explainability of our approach.</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Remix factors; reuse antecedents; online communities; creative work; songwriting; Songtree</t>
+          <t>Skill Recommendation; Explainable Recommendation; Reinforcement Learning; Deep Q Network; Case-based Reasoning; Prototype Learning; Self-Interpretable Neural Network</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr"/>
@@ -3289,7 +3131,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>521</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -3297,17 +3139,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Back to the Roots: Assessing Mining Techniques for Java Vulnerability-Contributing Commits</t>
+          <t>A Method to Analyze Multiple Social Identities in Twitter Bios</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Context: Vulnerability-contributing commits (VCCs) are code changes that introduce vulnerabilities. Mining historical VCCs relies on SZZ-based algorithms that trace from known vulnerability-fixing commits. Objective: Although these techniques have been used, e.g., to train just-in-time vulnerability predictors, they lack systematic benchmarking to evaluate their precision, recall, and error sources. Method: We empirically assessed 12 VCC mining techniques in Java repositories using two benchmark datasets (one from the literature and one newly curated). We also explored combinations of techniques, through intersections, voting schemes, and machine learning, to improve performance. Results: Individual techniques achieved at most 0.60 precision but up to 0.89 recall. The precision rose to 0.75 when the outputs were combined with the logical AND, at the expense of recall. Machine learning ensembles reached 0.80 precision with a better precision–recall balance. Performance varied significantly by dataset. Analyzing “fixing commits” showed that certain fix types (e.g., filtering or sanitization) affect retrieval accuracy, and failure patterns highlighted weaknesses when fixes involve external data handling. Conclusion: Such results help software security researchers select the most suitable mining technique for their studies and understand new ways to design more accurate solutions.</t>
+          <t>Twitter users signal social identity in their profile descriptions, or bios, in a number of important but complex ways that are not well-captured by existing characterizations of how identity is expressed in language. Better ways of defining and measuring these expressions may therefore be useful both in understanding how social identity is expressed in text, and how the self is presented on Twitter. To this end, the present work makes three contributions. First, using qualitative methods, we identify and define the concept of a personal identifier, which is more representative of the ways in which identity is signaled in Twitter bios. Second, we propose a method to extract all personal identifiers expressed in a given bio. Finally, we present a series of validation analyses that explore the strengths and limitations of our proposed method. Our work opens up exciting new opportunities at the intersection between the social psychological study of social identity and the study of how we compose the self through markers of identity on Twitter and in social media more generally.</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Mining Software Repositories; Software Vulnerability; Software Analytics; Machine Learning</t>
+          <t>computational social science; self-presentation; social identity; twitter</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
@@ -3330,7 +3172,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>567</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -3338,17 +3180,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Arising of Informal Women's Learn-to-code Communities: Activity Systems as Incubators</t>
+          <t>Understanding is a Two-Way Street: User-Initiated Repair on Agent Responses and Hearing in Conversational Interfaces</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Female-focused, grassroots communities purporting to help women learn to code are popping up in a variety of settings, indicating the motivation on the part of the participants to evade male-dominated settings while learning. However, little is known about how these groups function as an activity system. With current technology enabling the forming of virtual communities and the meteoric rise in use of the Salesforce CRM (customer relationship management) platform, a group of women have formed a coaching and learning community designed to help women move from Salesforce administrators to software developers through learning to code. We used activity systems analysis (ASA) to investigate this real-world instance of the larger phenomenon using an ethnographic approach. We used ASA to organize and make sense of the data by first creating a table listing the points on the activity system triangle (subject, rules, object, etc.) and filling in the points of the triangle based on the design of the coaching and learning group as described by participants; this gave us a high-level view of the activity system. To understand the subjects’ point of view of the system, we then created a new column in the table to fill in themes that emerged from our qualitative data analysis organized by dimension of the activity system. This process enabled us to capture the activity and the voices of participants as well as tensions that had emerged in the system. Findings show a range of outcomes, from participants crediting the group as a kickstart to the journey to successfully landing a job as a developer to members stalling in their progress after involvement. Results also show that purposeful tensions of welcoming novice questions and offering unsolicited verbal encouragement built into the activity system create a welcoming, safe environment for women learning to code.</t>
+          <t>Although methods for repairing prior turns in natural conversation are critical for enabling mutual understanding, or successful communication, these methods are seldom built into conversational user interfaces systematically. Chatbots and voice assistants tend to ask users to paraphrase what they said if it was not understood, but users cannot do the same if they encounter trouble in understanding what the agent said. Understanding is a one-way street in most (intent-based) conversation-like interfaces. An exception to this is Moore and Arar (2019), who demonstrate nine types of user-initiated repair on agent responses that are common in natural conversation and who have shown that users will employ these repair features correctly in text-based interfaces if taught. In this small-scale study, we test these user-initiated repairs (in second position) in a voice-based interface. With understanding-oriented repairs, we found that participants employed them much the same way in text and voice. In addition, we examine some hearing- and speaking-oriented repairs that emerged from the use of our novel multi-modal interface. We found that participants used them to manage troubles specific to the voice modality. Analysis of user logs and transcripts suggests that user-initiated repair features are valuable components of conversational interfaces.</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Informal learning; activity system; software development; women; workplace</t>
+          <t>chatbots; conversational agents; conversational ai; conversational user interfaces; conversational ux; user-initiated repair</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
@@ -3357,11 +3199,7 @@
           <t>EC5</t>
         </is>
       </c>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n"/>
       <c r="K71" s="2" t="n"/>
       <c r="L71" s="2" t="n"/>
@@ -3375,7 +3213,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>583</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -3383,17 +3221,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Designing Mid-Air Haptic Gesture Controlled User Interfaces for Cars</t>
+          <t>A Survey of Asynchronous Programming Using Coroutines in the Internet of Things and Embedded Systems</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>We present advancements in the design and development of in-vehicle infotainment systems that utilize gesture input and ultrasonic mid-air haptic feedback. Such systems employ state-of-the-art hand tracking technology and novel haptic feedback technology and promise to reduce driver distraction while performing a secondary task therefore cutting the risk of road accidents. In this paper, we document design process considerations during the development of a mid-air haptic gesture-enabled user interface for human-vehicle-interactions. This includes an online survey, business development insights, background research, and an agile framework component with three prototype iterations and user-testing on a simplified driving simulator. We report on the reasoning that led to the convergence of the chosen gesture-input and haptic-feedback sets used in the final prototype, discuss the lessons learned, and give hints and tips that act as design guidelines for future research and development of this technology in cars.</t>
+          <t>Many Internet of Things and embedded projects are event driven, and therefore require asynchronous and concurrent programming. Current proposals for C++20 suggest that coroutines will have native language support. It is timely to survey the current use of coroutines in embedded systems development. This article investigates existing research which uses or describes coroutines on resource-constrained platforms. The existing research is analysed with regard to: software platform, hardware platform, and capacity; use cases and intended benefits; and the application programming interface design used for coroutines. A systematic mapping study was performed, to select studies published between 2007 and 2018 which contained original research into the application of coroutines on resource-constrained platforms. An initial set of 566 candidate papers, collated from on-line databases, were reduced to only 35 after filters were applied, revealing the following taxonomy. The C 8 C++ programming languages were used by 22 studies out of 35. As regards hardware, 16 studies used 8- or 16-bit processors while 13 used 32-bit processors. The four most common use cases were concurrency (17 papers), network communication (15), sensor readings (9), and data flow (7). The leading intended benefits were code style and simplicity (12 papers), scheduling (9), and efficiency (8). A wide variety of techniques have been used to implement coroutines, including native macros, additional tool chain steps, new language features, and non-portable assembly language. We conclude that there is widespread demand for coroutines on resource-constrained devices. Our findings suggest that there is significant demand for a formalised, stable, well-supported implementation of coroutines in C++, designed with consideration of the special needs of resource-constrained devices, and further that such an implementation would bring benefits specific to such devices.</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>user experience design; ultrasound haptics; in-vehicle controls; human-machine interface; gesture interaction</t>
+          <t>scheduling; resource-constrained; direct style; asynchronous; Embedded</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
@@ -3416,7 +3254,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>59</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -3424,25 +3262,25 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Automatic API Usage Scenario Documentation from Technical Q&amp;amp;A Sites</t>
+          <t>Recruitment Promotion via Twitter: A Network-centric Approach of Analyzing Community Engagement Using Social Identity</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>The online technical Q&amp;amp;A site Stack Overflow (SO) is popular among developers to support their coding and diverse development needs. To address shortcomings in API official documentation resources, several research works have thus focused on augmenting official API documentation with insights (e.g., code examples) from SO. The techniques propose to add code examples/insights about APIs into its official documentation. Recently, surveys of software developers find that developers in SO consider the combination of code examples and reviews about APIs as a form of API documentation, and that they consider such a combination to be more useful than official API documentation when the official resources can be incomplete, ambiguous, incorrect, and outdated. Reviews are opinionated sentences with positive/negative sentiments. However, we are aware of no previous research that attempts to automatically produce API documentation from SO by considering both API code examples and reviews. In this article, we present two novel algorithms that can be used to automatically produce API documentation from SO by combining code examples and reviews towards those examples. The first algorithm is called statistical documentation, which shows the distribution of positivity and negativity around the code examples of an API using different metrics (e.g., star ratings). The second algorithm is called concept-based documentation, which clusters similar and conceptually relevant usage scenarios. An API usage scenario contains a code example, a textual description of the underlying task addressed by the code example, and the reviews (i.e., opinions with positive and negative sentiments) from other developers towards the code example. We deployed the algorithms in Opiner, a web-based platform to aggregate information about APIs from online forums. We evaluated the algorithms by mining all Java JSON-based posts in SO and by conducting three user studies based on produced documentation from the posts. The first study is a survey, where we asked the participants to compare our proposed algorithms against a Javadoc-syle documentation format (called as Type-based documentation in Opiner). The participants were asked to compare along four development scenarios (e.g., selection, documentation). The participants preferred our proposed two algorithms over type-based documentation. In our second user study, we asked the participants to complete four coding tasks using Opiner and the API official and informal documentation resources. The participants were more effective and accurate while using Opiner. In a subsequent survey, more than 80% of participants asked the Opiner documentation platform to be integrated into the formal API documentation to complement and improve the API official documentation.</t>
+          <t>With the proliferation of online technologies, social media recruitment has become an essential part of any company’s outreach campaign. A social media platform can provide marketing posts with access to a large pool of candidates and at a low cost. It also provides the opportunity to quickly customize and refine messages in response to the reception. With online marketing, the key question is: which communities are attracted by recruitment tweets on social media? In this work, we profile the Twitter accounts that interact with a set of recruitment tweets by the U.S. Army’s Recruitment Command through a network-centric perspective. By harnessing how users signal their affiliations through user information, we extract and analyze communities of social identities. From Social Identity Theory, these social identities can be critical drivers of behavior, like the decision to enlist in the military. With this framework, we evaluate the effectiveness of the U.S. Army’s recruitment campaign on Twitter, observing that these campaigns typically attract communities with military exposure like veterans or those that identify with professional careers and fitness (e.g., student, professionals, athletes). The campaign also attracts, but at a much lower level, interaction from those in the digital industries—data scientists, cybersecurity professionals, and so forth. When analyzing the accounts in terms of their degree of automation, we find a set of intent-unknown bot accounts interacting with the tweets, and that many of the recruitment accounts are perceived as automated accounts. These observations can aid in campaign refinement: targeting the digital community and getting a broader reach for online recruitment publicity campaigns.</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>usage scenario; documentation; crowd-sourced developer forum; API</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+          <t>Twitter; bot detection; network analysis; social signaling; social identity</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC2</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n"/>
       <c r="K73" s="2" t="n"/>
@@ -3457,7 +3295,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>629</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -3465,17 +3303,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Functional programming for modular Bayesian inference</t>
+          <t>SnappView, a Software Development Kit for Supporting End-user Mobile Interface Review</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>We present an architectural design of a library for Bayesian modelling and inference in modern functional programming languages. The novel aspect of our approach are modular implementations of existing state-of-the-art inference algorithms. Our design relies on three inherently functional features: higher-order functions, inductive data-types, and support for either type-classes or an expressive module system. We provide a performant Haskell implementation of this architecture, demonstrating that high-level and modular probabilistic programming can be added as a library in sufficiently expressive languages. We review the core abstractions in this architecture: inference representations, inference transformations, and inference representation transformers. We then implement concrete instances of these abstractions, counterparts to particle filters and Metropolis-Hastings samplers, which form the basic building blocks of our library. By composing these building blocks we obtain state-of-the-art inference algorithms: Resample-Move Sequential Monte Carlo, Particle Marginal Metropolis-Hastings, and Sequential Monte Carlo Squared. We evaluate our implementation against existing probabilistic programming systems and find it is already competitively performant, although we conjecture that existing functional programming optimisation techniques could reduce the overhead associated with the abstractions we use. We show that our modular design enables deterministic testing of inherently stochastic Monte Carlo algorithms. Finally, we demonstrate using OCaml that an expressive module system can also implement our design.</t>
+          <t>This paper presents SnappView, an open-source software development kit that facilitates end-user review of graphical user interfaces for mobile applications and streamlines their input into a continuous design life cycle. SnappView structures this user interface review process into four cumulative stages: (1) a developer creates a mobile application project with user interface code instrumented by only a few instructions governing SnappView and deploys the resulting application on an application store; (2) any tester, such as an end-user, a designer, a reviewer, while interacting with the instrumented user interface, shakes the mobile device to freeze and capture its screen and to provide insightful multimodal feedback such as textual comments, critics, suggestions, drawings by stroke gestures, voice or video records, with a level of importance; (3) the screenshot is captured with the application, browser, and status data and sent with the feedback to SnappView server; and (4) a designer then reviews collected and aggregated feedback data and passes them to the developer to address raised usability problems. Another cycle then initiates an iterative design. This paper presents the motivations and process for performing mobile application review based on SnappView. Based on this process, we deployed on the AppStore "WeTwo", a real-world mobile application to find various personal activities over a one-month period with 420 active users. This application served for a user experience evaluation conducted with N1=14 developers to reveal the advantages and shortcomings of the toolkit from a development point of view. The same application was also used in a usability evaluation conducted with N2=22 participants to reveal the advantages and shortcomings from an end-user viewpoint.</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>type-classes; probabilistic programming; monads; monad transformers; module systems; machine learning; inductive types; higher-order functions; functional programming; WebPPL; Sequential Monte Carlo; Monte Carlo samplers; Markov Chain Monte Carlo; Bayesian inference; Anglican</t>
+          <t>GUI testing; application review; code instrumentation; heuristic evaluation; mobile computing; remote evaluation; software development kit; usability evaluation; usability problem; user interface evaluation</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
@@ -3498,7 +3336,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -3506,15 +3344,19 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Teaching embedded systems using the raspberry PI and sense hat</t>
+          <t>An Architectural Viewpoint for Benefit-Cost-Risk-Aware Decision-Making in Self-Adaptive Systems</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>This paper describes an upper division course in embedded systems development for Computer Science majors who have not had any Engineering courses. The course was developed to teach low-level programming, sensors, and some real-time concepts; using the Raspberry Pi™ and the Sense HAT™ sensor platform; with Python and C as programming languages.</t>
-        </is>
-      </c>
-      <c r="F75" s="3" t="inlineStr"/>
+          <t>Self-adaptation equips a software system with a feedback loop that resolves uncertainties during operation and adapts the system to deal with them when necessary. Most self-adaptation approaches today use decision-making mechanisms that select for execution the adaptation option with the best-estimated benefit expressed as a set of adaptation goals. A few approaches also consider the estimated (one-off) cost of executing the candidate adaptation options. We argue that besides benefit and cost, decision-making in self-adaptive systems should also consider the estimated risk the system or its users would be exposed to if an adaptation option were selected for execution. Balancing all three concerns when evaluating the options for adaptation to mitigate uncertainty is essential for satisfying stakeholders’ concerns and ensuring the safety and public acceptance of self-adaptive systems. In this article, we present a reference model for decision-making in self-adaptation that considers the estimated benefit, cost, and risk as core concerns of each adaptation option. Leveraging this model, we then present an ISO/IEC/IEEE 42010 compatible architectural viewpoint that aims at supporting software architects responsible for designing robust decision-making mechanisms for self-adaptive systems. We demonstrate the applicability, usefulness, and understandability of the viewpoint through a case study where participants with experience in the engineering of self-adaptive systems performed a set of design tasks in DeltaIoT, an Internet-of-Things exemplar for research on self-adaptive systems.</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>self-adaptive; risk; cost; benefit; viewpoint; decision-making</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3535,7 +3377,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>604</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -3543,17 +3385,17 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>An empirical comparison of formalisms for modelling and analysis of dynamic reconfiguration of dependable systems</t>
+          <t>Adventures in monitorability: from branching to linear time and back again</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>This paper uses a case study to evaluate empirically three formalisms of different kinds for their suitability for the modelling and analysis of dynamic reconfiguration of dependable systems. The requirements on an ideal formalism for dynamic software reconfiguration are defined. The reconfiguration of an office workflow for order processing is described, and the requirements on the reconfiguration of the workflow are defined. The workflow is modelled using the Vienna Development Method (VDM), conditional partial order graphs (CPOGs), and the basic Calculus of Communicating Systems for dynamic process reconfiguration (basic CCSdp), and verification of the reconfiguration requirements is attempted using the models. The formalisms are evaluated according to their ability to model the reconfiguration of the workflow, to verify the requirements on the workflow’s reconfiguration, and to meet the requirements on an ideal formalism.</t>
+          <t>This paper establishes a comprehensive theory of runtime monitorability for Hennessy-Milner logic with recursion, a very expressive variant of the modal µ-calculus. It investigates the monitorability of that logic with a linear-time semantics and then compares the obtained results with ones that were previously presented in the literature for a branching-time setting. Our work establishes an expressiveness hierarchy of monitorable fragments of Hennessy-Milner logic with recursion in a linear-time setting and exactly identifies what kinds of guarantees can be given using runtime monitors for each fragment in the hierarchy. Each fragment is shown to be complete, in the sense that it can express all properties that can be monitored under the corresponding guarantees. The study is carried out using a principled approach to monitoring that connects the semantics of the logic and the operational semantics of monitors. The proposed framework supports the automatic, compositional synthesis of correct monitors from monitorable properties.</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Basic CCSdp; Conditional partial order graphs; VDM; Formal methods; Reconfiguration requirements; Workflow case study; Dynamic software reconfiguration</t>
+          <t>monitorability; monitor synthesis; linear-time and branching-time logics</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
@@ -3576,7 +3418,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>692</t>
+          <t>674</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -3584,17 +3426,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Incrementalizing lattice-based program analyses in Datalog</t>
+          <t>Continuous and Proactive Software Architecture Evaluation: An IoT Case</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Program analyses detect errors in code, but when code changes frequently as in an IDE, repeated re-analysis from-scratch is unnecessary: It leads to poor performance unless we give up on precision and recall. Incremental program analysis promises to deliver fast feedback without giving up on precision or recall by deriving a new analysis result from the previous one. However, Datalog and other existing frameworks for incremental program analysis are limited in expressive power: They only support the powerset lattice as representation of analysis results, whereas many practically relevant analyses require custom lattices and aggregation over lattice values. To this end, we present a novel algorithm called DRedL that supports incremental maintenance of recursive lattice-value aggregation in Datalog. The key insight of DRedL is to dynamically recognize increasing replacements of old lattice values by new ones, which allows us to avoid the expensive deletion of the old value. We integrate DRedL into the analysis framework IncA and use IncA to realize incremental implementations of strong-update points-to analysis and string analysis for Java. As our performance evaluation demonstrates, both analyses react to code changes within milliseconds.</t>
+          <t>Design-time evaluation is essential to build the initial software architecture to be deployed. However, experts’ assumptions made at design-time are unlikely to remain true indefinitely in systems that are characterized by scale, hyperconnectivity, dynamism, and uncertainty in operations (e.g. IoT). Therefore, experts’ design-time decisions can be challenged at run-time. A continuous architecture evaluation that systematically assesses and intertwines design-time and run-time decisions is thus necessary. This paper proposes the first proactive approach to continuous architecture evaluation of the system leveraging the support of simulation. The approach evaluates software architectures by not only tracking their performance over time, but also forecasting their likely future performance through machine learning of simulated instances of the architecture. This enables architects to make cost-effective informed decisions on potential changes to the architecture. We perform an IoT case study to show how machine learning on simulated instances of architecture can fundamentally guide the continuous evaluation process and influence the outcome of architecture decisions. A series of experiments is conducted to demonstrate the applicability and effectiveness of the approach. We also provide the architect with recommendations on how to best benefit from the approach through choice of learners and input parameters, grounded on experimentation and evidence.</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Static Analysis; Lattice; Language Workbench; Incremental Computing; Domain-Specific Language; Datalog</t>
+          <t>Continuous evaluation; software architecture evaluation; time series forecasting; IoT</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr"/>
@@ -3617,7 +3459,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>678</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -3625,30 +3467,26 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>How Configurable Is the Linux Kernel? Analyzing Two Decades of Feature-Model History</t>
+          <t>Incentive Mechanisms for Participatory Sensing: Survey and Research Challenges</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Today, the operating system Linux is widely used in diverse environments, as its kernel can be configured flexibly. In many configurable systems, managing such variability can be facilitated in all development phases with product-line analyses. These analyses often require knowledge about the system’s features and their dependencies, which are documented in a feature model. Despite their potential, product-line analyses are rarely applied to the Linux kernel in practice, as its feature model still challenges scalability and accuracy of analyses. Unfortunately, these challenges also severely limit our knowledge about two fundamental metrics of the kernel’s configurability, namely its number of features and configurations. We identify four key limitations in the literature related to the scalability, accuracy, and influence factors of these metrics, and, by extension, other product-line analyses: (1) Analysis results for the Linux kernel are not comparable, because relevant information is not reported; (2) there is no consensus on how to define features in Linux, which leads to flawed analysis results; (3) only few versions of the Linux kernel have ever been analyzed, none of which are recent; and (4) the kernel is perceived as complex, although we lack empirical evidence that supports this claim. In this article, we address these limitations with a comprehensive, empirical study of the Linux kernel’s configurability, which spans its feature model’s entire history from 2002 to 2024. We address the above limitations as follows: (1) We characterize parameters that are relevant when reporting analysis results; (2) we propose and evaluate a novel definition of features in Linux as a standardization effort; (3) we contribute torte, a tool that analyzes arbitrary versions of the Linux kernel’s feature model; and (4) we investigate the current and possible future configurability of the kernel on more than 3,000 feature-model versions. Based on our results, we highlight 11 major insights into the Linux kernel’s configurability and make 7 actionable recommendations for researchers and practitioners.</t>
+          <t>Participatory sensing is a powerful paradigm that takes advantage of smartphones to collect and analyze data beyond the scale of what was previously possible. Given that participatory sensing systems rely completely on the users’ willingness to submit up-to-date and accurate information, it is paramount to effectively incentivize users’ active and reliable participation. In this article, we survey existing literature on incentive mechanisms for participatory sensing systems. In particular, we present a taxonomy of existing incentive mechanisms for participatory sensing systems, which are subsequently discussed in depth by comparing and contrasting different approaches. Finally, we discuss an agenda of open research challenges in incentivizing users in participatory sensing.</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Linux kernel; feature modeling; software product lines; software variability</t>
+          <t>survey; research challenges; game theory; auction theory; QoI</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>EC4</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+          <t>EC5</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="n"/>
       <c r="K78" s="2" t="n"/>
       <c r="L78" s="2" t="n"/>
@@ -3662,7 +3500,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>683</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -3670,30 +3508,26 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Identifying Non-Technical Skill Gaps in Software Engineering Education: What Experts Expect But Students Don’t Learn</t>
+          <t>odeToJava: A PSE for the Numerical Solution of IVPs</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>As the importance of non-technical skills in the software engineering industry increases, the skill sets of graduates match less and less with industry expectations. A growing body of research exists that attempts to identify this skill gap. However, only few so far explicitly compare opinions of the industry with what is currently being taught in academia. By aggregating data from three previous works, we identify the three biggest non-technical skill gaps between industry and academia for the field of software engineering: devoting oneself to continuous learning, being creative by approaching a problem from different angles, and thinking in a solution-oriented way by favoring outcome over ego. Eight follow-up interviews were conducted to further explore how the industry perceives these skill gaps, yielding 26 sub-themes grouped into six bigger themes: stimulating continuous learning, stimulating creativity, creative techniques, addressing the gap in education, skill requirements in industry, and the industry selection process. With this work, we hope to inspire educators to give the necessary attention to the uncovered skills, further mitigating the gap between the industry and the academic world.</t>
+          <t>Problem-solving environments (PSEs) offer a powerful yet flexible and convenient means for general experimentation with computational methods, algorithm prototyping, and visualization and manipulation of data. Consequently, PSEs have become the modus operandi of many computational scientists and engineers. However, despite these positive aspects, PSEs typically do not offer the level of granularity required by the specialist or algorithm designer to conveniently modify the details. In other words, the level at which PSEs are black boxes is often still too high for someone interested in modifying an algorithm as opposed to trying an alternative.In this article, we describe odeToJava, a Java-based PSE for initial-value problems in ordinary differential equations. odeToJava implements explicit and linearly implicit implicit-explicit Runge--Kutta methods with error and stepsize control and intra-step interpolation (dense output), giving the user control and flexibility over the implementational aspects of these methods. We illustrate the usage and functionality of odeToJava by means of computational case studies of initial-value problems (IVPs).</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Software engineering education; creativity; professional skills; software developer; industry requirements</t>
+          <t>Adaptive integration; Runge--Kutta; St\"{o}rmer--Verlet; additive Runge--Kutta; geometric integration; object-oriented; problem solving environment; software architecture; stepsize-control</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>EC5</t>
-        </is>
-      </c>
-      <c r="I79" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>EC4</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n"/>
       <c r="K79" s="2" t="n"/>
       <c r="L79" s="2" t="n"/>
@@ -3702,12 +3536,12 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Scopus</t>
+          <t>ACM Digital Library</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>79</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -3715,30 +3549,26 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>A Job Finder Chatbot-Based Web Platform: A Use Case for Software Engineers</t>
+          <t>RAPID: Zero-Shot Domain Adaptation for Code Search with Pre-Trained Models</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Finding a job requires browsing through a vast number of position openings, usually at various online sites. This process becomes more complicated for users when they are considering different potential job locations. Even though existing tools that automate the process exist (e.g. sonara.ai, dream.jobs), they lack the element of interactivity with the user and the integration of external resources that contain information on the skills of the user. With the aim to bridge the gap between job seekers and potential employers by matching resumes and job listings more efficiently and effectively, in this work we are introducing an AI-driven chatbot-based web platform to assist job seeking. In the initial implementation, we are considering the job seeking needs of software engineers but more disciplines can be easily added. We have integrated the developer's CV and the user's GitHub account, and are describing the design and implementation process of the web platform, while a small scale user evaluation has also been performed. We argue that the chatbot can be used as a starting point for similar job seeking assistants. Copyright © 2025 by SCITEPRESS - Science and Technology Publications, Lda.</t>
+          <t>Code search, which refers to the process of identifying the most relevant code snippets for a given natural language query, plays a crucial role in software maintenance. However, current approaches heavily rely on labeled data for training, which results in performance decreases when confronted with cross-domain scenarios including domain- or project-specific situations. This decline can be attributed to their limited ability to effectively capture the semantics associated with such scenarios. To tackle the aforementioned problem, we propose a zeRo-shot domAin adaPtion with pre-traIned moDels framework for code search named RAPID. The framework first generates synthetic data by pseudo labeling, then trains the CodeBERT with sampled synthetic data. To avoid the influence of noisy synthetic data and enhance the model performance, we propose a mixture sampling strategy to obtain hard negative samples during training. Specifically, the mixture sampling strategy considers both relevancy and diversity to select the data that are hard to be distinguished by the models. To validate the effectiveness of our approach in zero-shot settings, we conduct extensive experiments and find that RAPID outperforms the CoCoSoDa and UniXcoder model by an average of 15.7% and 10%, respectively, as measured by the MRR metric. When trained on full data, our approach results in an average improvement of 7.5% under the MRR metric using CodeBERT. We observe that as the model’s performance in zero-shot tasks improves, the impact of hard negatives diminishes. Our observation also indicates that fine-tuning CodeT5 for generating pseudo labels can enhance the performance of the code search model, and using only 100-shot samples can yield comparable results to the supervised baseline. Furthermore, we evaluate the effectiveness of RAPID in real-world code search tasks in three GitHub projects through both human and automated assessments. Our findings reveal RAPID exhibits superior performance, e.g., an average improvement of 18% under the MRR metric over the top-performing model.</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Chatbots; Employment; Information systems; Information use; Knowledge management; Software engineering; Websites; Chatbots; Engineering position; Github; Hard skill; Interactivity; Job advert; Job-seeking; Online sites; Soft skills; Software engineering position; Engineers</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>IC2; IC5</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr"/>
-      <c r="I80" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>Code search; zero-shot learning; software maintenance; pre-trained models; domain adaption</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n"/>
       <c r="K80" s="2" t="n"/>
       <c r="L80" s="2" t="n"/>
@@ -3747,12 +3577,12 @@
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Scopus</t>
+          <t>IEEE Xplore</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>833</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -3760,17 +3590,17 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Validating a Set of Candidate Criteria for Evaluating Software Tools and Data Sources for National CSIRTs’ Cyber Incident Responses</t>
+          <t>IEEE Magazines</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>National Computer Security Incident Response Teams (CSIRTs) are established worldwide to coordinate responses to cyber security incidents at the national level. It is known that software tools (including open source ones) and public data are routinely used to facilitate incident response in national CSIRTs. However, there is a lack of an authoritative set of criteria that can be used for a systematic evaluation to decide which software tools and data sources should be used by national CSIRTs for incident response. A prior study identified a set of potential candidate criteria for such an evaluation. The study presented in this article aims to validate these candidate criteria empirically by asking staff members of several national CSIRTs how they perceive the candidate criteria’s practical usefulness and readiness for deployment in national CSIRTs’ operations. The study involved online semi-structured interviews with nine interviewees from nine national CSIRTs in Asia-Pacific, Africa and Europe. After validating the candidate criteria using semi-structured interviews with these nine interviewees, we applied the criteria to evaluate a selection of software tools and data sources by converting each criterion into one or more relevant metrics, such as ‘measuring the time taken by a tool to produce results’. Results from the study led to the following main findings: (1) all interviewees perceived the candidate criteria as practically useful for evaluating tools and data sources in the operations of national CSIRTs; (2) all interviewees agreed that the candidate criteria could be deployed in national CSIRTs and other types of CSIRTs and (3) the candidate criteria can be applied relatively easily in practice. These criteria are envisaged to help national CSIRTs select the most appropriate tools and data sources to facilitate effective incident response, improve their operational practices and improve the quality of wider security operations. © 2025 Copyright held by the owner/author(s).</t>
+          <t>A major concern among graduates of computing departments is the discrepancy between the expectations of software companies and the competencies provided by the academic departments. This ongoing problem makes co-op education inevitable, as it combines industrial experience with traditional education.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Computer aided software engineering; Computer software selection and evaluation; National security; Network security; Open systems; Security systems; CERT; Computer security incident response team; Criteria; Cybe incident response; Data evaluation; Incident response; National computer security incident response team; Security incident; Semi structured interviews; Tools evaluations; Open source software</t>
+          <t>Companies; Education; Employment; Software engineering; Recruitment; Software; Training; Computer science education; Educational courses; Career development</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr"/>
@@ -3793,7 +3623,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>994</t>
+          <t>927</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -3801,26 +3631,26 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Recruitment in SMEs: the role of managerial practices, technology and innovation</t>
+          <t>Desired Qualifications Sought in Entry Level Software Engineers</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Purpose: Various scholars suggest that there is a lack of research on the recruitment in small and medium-sized enterprises (SMEs) and also a scarcity of theoretical basis for the recruitment procedures used by these companies. As the vast majority of studies concentrate on larger organizations, they may not accurately reflect the challenges faced by smaller-sized entities to profoundly and accurately comprehend their recruitment procedures. In addition, the use of technology in recruitment has grown in importance in today’s quickly evolving business environment, particularly in light of the COVID-19 pandemic footprint. This study aims to examine the recruitment procedures used by SMEs and how they have been compelled to adjust to different extents to these technological improvements by the effects of the aforementioned epidemic. Design/methodology/approach: With the aim to investigate the current recruitment practices in SMEs and the extent to which digital technologies are embraced by these companies within human resources (HR) procedures, this research relied on interviews with SMEs representatives. The qualitative methods used provided access to relevant data and insights, as they allowed close interactions with top managers and CEOs of ten companies from various sectors. Thus, the research results draw a vivid and reliable image of the procedures and practices used by small and medium-sized companies to attract, select and retain their staff. Findings: This study’s findings are of increased interest to HR professionals, recruiters and managers in SMEs, who aim to attract and retain the best talent and optimize their recruitment strategies in a rapidly changing business environment, enabled by technological advancements. Effective HR recruitment procedures adapted to the specific needs of small and medium-sized companies can lead to several benefits for the organization, including improved employee selection, reduced turnover and increased organizational productivity. Research limitations/implications: Although the interviews examined here encompass recruitment techniques from SMEs in a variety of industries, the results’ generalizability is limited by the sample size and geography. Furthermore, the findings’ dependability is dependent on the accuracy of the data provided by the respondents. Practical implications: This investigation confirms some of the theoretical underpinnings which point to the lack of formalized structures and procedures in the recruitment process in SMEs, which enjoy more flexibility in managing HR processes. In addition, the results reinforce the arguments indicating an adjustment between HR strategies or policies and organizational goals in smaller enterprises which adapt faster to changes in the market. Moreover, it becomes apparent that there is a relationship between the quality of job descriptions and the successful fit in attracting the right candidates for the open positions. Furthermore, digital technologies offer opportunities for expanding the recruiters’ reach to a wider audience and also support the selection stage, thus increasing the chances of finding suitable staff. As the need to shift from traditional recruitment to e-recruitment in SMEs has been highlighted in the literature, the qualitative research revealed that this need was driven on the one hand by the COVID-19 pandemic when these companies successfully adapted and implemented new online methods of recruiting, but also by the lack of skilled labor, leading to the expansion of recruitment to other parts of the country or even to other countries. Social implications: With regard to the proportion of men and women used in small and medium-sized companies, there is a clear need to involve and train more women in the predominantly male-dominated industrial and IT sectors. From this point of view, companies tend to devote more interest to integrating communities of women in these industries, as well as in key management positions. Another point of interest that the study highlights is the fact that SMEs have started to get creative with the benefits package they propose to candidates and focus on remote work, hybrid office–home working, or seasonal work to offer future employees a better work–life balance. Originality/value: The added value of this investigation is filling the gaps in the current literature concerning recruitment procedures currently used by SMEs, the challenges they face and the solutions they advanced to solve them. Furthermore, SMEs often drive innovation and competition in the market and play a crucial role in the supply chain of larger companies, providing them with the goods and services they need to operate and supporting the availability and reliability of products from larger companies. They are often the driving force behind revitalizing local economies and creating new employment opportunities. Consequently, the underlying significance of this study is rooted in the need to modernize and simultaneously improve HR recruitment procedures through the integration of technology and a focus on innovation. © 2023, Emerald Publishing Limited.</t>
-        </is>
-      </c>
-      <c r="F82" s="3" t="inlineStr"/>
+          <t>Global demand for software engineers continues to strain the technology sector with unfilled software engineering positions and stiff competition for hiring developers who are on the market. To attract more candidates, technology firms have increasingly been working closely with universities to recruit new graduates to fill their jobs. Universities hoping to minimize mismatches in job placement for new software developers should teach the skills and attributes that enable entry-level software developers to succeed. This paper presents a case study of hiring demands at one large, well-established technology company that reveals the most sought-after attributes in new hires. We discuss results of our interviews with five software development hiring managers and the results from a wide survey of engineers and architects from various levels and experiences. The interviews and surveys reveal that some qualifications are widely desired, and others have varying demand based on functional area, technology, or type of development. Ultimately, professional skills (e.g., teamwork) and personality traits (e.g., strong initiative) top the list of desired attributes, along with a few fundamentally broad technical skills. One key takeaway is that candidates who learn professional skills from university programs may be more readily hired into their first software engineering job than those whose education focused mostly on technical areas. © 2023 ACM.</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Employment; Engineering education; Professional aspects; Software design; Case-studies; Employer-seek skill; Engineering position; Global demand; Hireability; Hiring managers; Professional skills; Software developer; Technology companies; Technology sectors; Engineers</t>
+        </is>
+      </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>IC1; IC2</t>
+          <t>IC1; IC4</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
-      <c r="I82" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="n"/>
       <c r="K82" s="2" t="n"/>
       <c r="L82" s="2" t="n"/>
@@ -3838,7 +3668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3868,8 +3698,8 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="6" t="n"/>
-      <c r="B2" s="6" t="n"/>
+      <c r="A2" s="4" t="n"/>
+      <c r="B2" s="4" t="n"/>
       <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Revisor 1</t>
@@ -3880,7 +3710,7 @@
           <t>Revisor 2</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n"/>
+      <c r="E2" s="4" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -3888,12 +3718,246 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Software Engineering Job Market: Salaries, Trends &amp; Insights</t>
+          <t>Software Engineering | Future Students</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Why are entry-level data and software engineering roles so ...</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Machine Learning with System/Software Engineering in ...</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Relationship between computer science and software ...</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>AI and Software Engineering: A Symbiotic Relationship</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Does familiarity with the attraction matter? Antecedents of ...</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>I am really into computers and I would love to study ...</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Tests - Pre-Employment ...</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Levels and Titles</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Gartner for Software Engineering Leaders</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Information technology Review 1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Reliability assessment of AI systems - ISO/IEC AWI TS 25570</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sampling in Software Engineering Research:A Critical Review ...</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Computer Programming and Analysis (Software Engineering ...</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>37 Hybrid &amp; Onsite Software Engineering Jobs in Tallinn ...</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Archives</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Information and Software Technology Journal</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Course - Career Choices &amp; Jobs</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>A Preliminary Guide for Assertive Selection of Active ...</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
feat(core): crossref integration, dynamic throttling, and dual prompting
</commit_message>
<xml_diff>
--- a/data/processed/export/APOLLO_Screening_Results.xlsx
+++ b/data/processed/export/APOLLO_Screening_Results.xlsx
@@ -661,7 +661,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -706,7 +706,7 @@
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -735,12 +735,12 @@
           <t>Data visualization; Visualization; API; Coding platform; Data; Digital resumes; Problem-solving; Project efficiency; Retrieval; Silicon valley; Software developer; Web scrapings; Websites</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC2</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -751,7 +751,7 @@
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -796,7 +796,7 @@
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -837,7 +837,7 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -866,12 +866,12 @@
           <t>collaborative and social computing; large language models; social simulation</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC2; IC4</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -882,7 +882,7 @@
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -919,7 +919,7 @@
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -956,7 +956,7 @@
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -993,7 +993,7 @@
       <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1030,7 +1030,7 @@
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -1075,7 +1075,7 @@
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
     </row>
-    <row r="12" ht="20" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1112,7 +1112,7 @@
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1149,7 +1149,7 @@
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1186,7 +1186,7 @@
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1">
+    <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1223,7 +1223,7 @@
       <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
     </row>
-    <row r="16" ht="20" customHeight="1">
+    <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1260,7 +1260,7 @@
       <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="n"/>
     </row>
-    <row r="17" ht="20" customHeight="1">
+    <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1297,7 +1297,7 @@
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1334,7 +1334,7 @@
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
     </row>
-    <row r="19" ht="20" customHeight="1">
+    <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1371,7 +1371,7 @@
       <c r="L19" s="2" t="n"/>
       <c r="M19" s="2" t="n"/>
     </row>
-    <row r="20" ht="20" customHeight="1">
+    <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1408,7 +1408,7 @@
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
     </row>
-    <row r="21" ht="20" customHeight="1">
+    <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1445,7 +1445,7 @@
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="n"/>
     </row>
-    <row r="22" ht="20" customHeight="1">
+    <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1482,7 +1482,7 @@
       <c r="L22" s="2" t="n"/>
       <c r="M22" s="2" t="n"/>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1519,7 +1519,7 @@
       <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="n"/>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1556,7 +1556,7 @@
       <c r="L24" s="2" t="n"/>
       <c r="M24" s="2" t="n"/>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -1601,7 +1601,7 @@
       <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="n"/>
     </row>
-    <row r="26" ht="20" customHeight="1">
+    <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1638,7 +1638,7 @@
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="n"/>
     </row>
-    <row r="27" ht="20" customHeight="1">
+    <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1675,7 +1675,7 @@
       <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="n"/>
     </row>
-    <row r="28" ht="20" customHeight="1">
+    <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1712,7 +1712,7 @@
       <c r="L28" s="2" t="n"/>
       <c r="M28" s="2" t="n"/>
     </row>
-    <row r="29" ht="20" customHeight="1">
+    <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1749,7 +1749,7 @@
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
     </row>
-    <row r="30" ht="20" customHeight="1">
+    <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1786,7 +1786,7 @@
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
     </row>
-    <row r="31" ht="20" customHeight="1">
+    <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1823,7 +1823,7 @@
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
     </row>
-    <row r="32" ht="20" customHeight="1">
+    <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1860,7 +1860,7 @@
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="n"/>
     </row>
-    <row r="33" ht="20" customHeight="1">
+    <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1897,7 +1897,7 @@
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="2" t="n"/>
     </row>
-    <row r="34" ht="20" customHeight="1">
+    <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1934,7 +1934,7 @@
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="n"/>
     </row>
-    <row r="35" ht="20" customHeight="1">
+    <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -1971,7 +1971,7 @@
       <c r="L35" s="2" t="n"/>
       <c r="M35" s="2" t="n"/>
     </row>
-    <row r="36" ht="20" customHeight="1">
+    <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2008,7 +2008,7 @@
       <c r="L36" s="2" t="n"/>
       <c r="M36" s="2" t="n"/>
     </row>
-    <row r="37" ht="20" customHeight="1">
+    <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2045,7 +2045,7 @@
       <c r="L37" s="2" t="n"/>
       <c r="M37" s="2" t="n"/>
     </row>
-    <row r="38" ht="20" customHeight="1">
+    <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2082,7 +2082,7 @@
       <c r="L38" s="2" t="n"/>
       <c r="M38" s="2" t="n"/>
     </row>
-    <row r="39" ht="20" customHeight="1">
+    <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2119,7 +2119,7 @@
       <c r="L39" s="2" t="n"/>
       <c r="M39" s="2" t="n"/>
     </row>
-    <row r="40" ht="20" customHeight="1">
+    <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2156,7 +2156,7 @@
       <c r="L40" s="2" t="n"/>
       <c r="M40" s="2" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1">
+    <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2193,7 +2193,7 @@
       <c r="L41" s="2" t="n"/>
       <c r="M41" s="2" t="n"/>
     </row>
-    <row r="42" ht="20" customHeight="1">
+    <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2230,7 +2230,7 @@
       <c r="L42" s="2" t="n"/>
       <c r="M42" s="2" t="n"/>
     </row>
-    <row r="43" ht="20" customHeight="1">
+    <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2267,7 +2267,7 @@
       <c r="L43" s="2" t="n"/>
       <c r="M43" s="2" t="n"/>
     </row>
-    <row r="44" ht="20" customHeight="1">
+    <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2304,7 +2304,7 @@
       <c r="L44" s="2" t="n"/>
       <c r="M44" s="2" t="n"/>
     </row>
-    <row r="45" ht="20" customHeight="1">
+    <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2349,7 +2349,7 @@
       <c r="L45" s="2" t="n"/>
       <c r="M45" s="2" t="n"/>
     </row>
-    <row r="46" ht="20" customHeight="1">
+    <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2386,7 +2386,7 @@
       <c r="L46" s="2" t="n"/>
       <c r="M46" s="2" t="n"/>
     </row>
-    <row r="47" ht="20" customHeight="1">
+    <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2407,12 +2407,12 @@
       </c>
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC3; IC5</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
           <t>YES</t>
@@ -2423,7 +2423,7 @@
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="n"/>
     </row>
-    <row r="48" ht="20" customHeight="1">
+    <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2460,7 +2460,7 @@
       <c r="L48" s="2" t="n"/>
       <c r="M48" s="2" t="n"/>
     </row>
-    <row r="49" ht="20" customHeight="1">
+    <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2497,7 +2497,7 @@
       <c r="L49" s="2" t="n"/>
       <c r="M49" s="2" t="n"/>
     </row>
-    <row r="50" ht="20" customHeight="1">
+    <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Springer Nature</t>
@@ -2534,7 +2534,7 @@
       <c r="L50" s="2" t="n"/>
       <c r="M50" s="2" t="n"/>
     </row>
-    <row r="51" ht="20" customHeight="1">
+    <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Web of Science</t>
@@ -2563,12 +2563,12 @@
           <t>Organizations; Project management; Recruitment; Software; Uncertainty; Stakeholders; Receivers; Agile project management (APM); Agile project manager (AgPM); competencies; job advertisements; signaling theory</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC2; IC3</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr">
         <is>
           <t>YES</t>
@@ -2579,7 +2579,7 @@
       <c r="L51" s="2" t="n"/>
       <c r="M51" s="2" t="n"/>
     </row>
-    <row r="52" ht="20" customHeight="1">
+    <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Web of Science</t>
@@ -2608,12 +2608,12 @@
           <t>Open Source Software; Mining Software Repositories; Developer Expertise; Visualization Tool</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC2; IC3</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>EC4</t>
+        </is>
+      </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2624,7 +2624,7 @@
       <c r="L52" s="2" t="n"/>
       <c r="M52" s="2" t="n"/>
     </row>
-    <row r="53" ht="20" customHeight="1">
+    <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2669,7 +2669,7 @@
       <c r="L53" s="2" t="n"/>
       <c r="M53" s="2" t="n"/>
     </row>
-    <row r="54" ht="20" customHeight="1">
+    <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2714,7 +2714,7 @@
       <c r="L54" s="2" t="n"/>
       <c r="M54" s="2" t="n"/>
     </row>
-    <row r="55" ht="20" customHeight="1">
+    <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2759,7 +2759,7 @@
       <c r="L55" s="2" t="n"/>
       <c r="M55" s="2" t="n"/>
     </row>
-    <row r="56" ht="20" customHeight="1">
+    <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2804,7 +2804,7 @@
       <c r="L56" s="2" t="n"/>
       <c r="M56" s="2" t="n"/>
     </row>
-    <row r="57" ht="20" customHeight="1">
+    <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2849,7 +2849,7 @@
       <c r="L57" s="2" t="n"/>
       <c r="M57" s="2" t="n"/>
     </row>
-    <row r="58" ht="20" customHeight="1">
+    <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2894,7 +2894,7 @@
       <c r="L58" s="2" t="n"/>
       <c r="M58" s="2" t="n"/>
     </row>
-    <row r="59" ht="20" customHeight="1">
+    <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2939,7 +2939,7 @@
       <c r="L59" s="2" t="n"/>
       <c r="M59" s="2" t="n"/>
     </row>
-    <row r="60" ht="20" customHeight="1">
+    <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -2984,7 +2984,7 @@
       <c r="L60" s="2" t="n"/>
       <c r="M60" s="2" t="n"/>
     </row>
-    <row r="61" ht="20" customHeight="1">
+    <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3029,7 +3029,7 @@
       <c r="L61" s="2" t="n"/>
       <c r="M61" s="2" t="n"/>
     </row>
-    <row r="62" ht="20" customHeight="1">
+    <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3074,7 +3074,7 @@
       <c r="L62" s="2" t="n"/>
       <c r="M62" s="2" t="n"/>
     </row>
-    <row r="63" ht="20" customHeight="1">
+    <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3119,7 +3119,7 @@
       <c r="L63" s="2" t="n"/>
       <c r="M63" s="2" t="n"/>
     </row>
-    <row r="64" ht="20" customHeight="1">
+    <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3160,7 +3160,7 @@
       <c r="L64" s="2" t="n"/>
       <c r="M64" s="2" t="n"/>
     </row>
-    <row r="65" ht="20" customHeight="1">
+    <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3205,7 +3205,7 @@
       <c r="L65" s="2" t="n"/>
       <c r="M65" s="2" t="n"/>
     </row>
-    <row r="66" ht="20" customHeight="1">
+    <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3250,7 +3250,7 @@
       <c r="L66" s="2" t="n"/>
       <c r="M66" s="2" t="n"/>
     </row>
-    <row r="67" ht="20" customHeight="1">
+    <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3295,7 +3295,7 @@
       <c r="L67" s="2" t="n"/>
       <c r="M67" s="2" t="n"/>
     </row>
-    <row r="68" ht="20" customHeight="1">
+    <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3340,7 +3340,7 @@
       <c r="L68" s="2" t="n"/>
       <c r="M68" s="2" t="n"/>
     </row>
-    <row r="69" ht="20" customHeight="1">
+    <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3385,7 +3385,7 @@
       <c r="L69" s="2" t="n"/>
       <c r="M69" s="2" t="n"/>
     </row>
-    <row r="70" ht="20" customHeight="1">
+    <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3430,7 +3430,7 @@
       <c r="L70" s="2" t="n"/>
       <c r="M70" s="2" t="n"/>
     </row>
-    <row r="71" ht="20" customHeight="1">
+    <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3475,7 +3475,7 @@
       <c r="L71" s="2" t="n"/>
       <c r="M71" s="2" t="n"/>
     </row>
-    <row r="72" ht="20" customHeight="1">
+    <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>ACM Digital Library</t>
@@ -3520,7 +3520,7 @@
       <c r="L72" s="2" t="n"/>
       <c r="M72" s="2" t="n"/>
     </row>
-    <row r="73" ht="20" customHeight="1">
+    <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -3565,7 +3565,7 @@
       <c r="L73" s="2" t="n"/>
       <c r="M73" s="2" t="n"/>
     </row>
-    <row r="74" ht="20" customHeight="1">
+    <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -3606,7 +3606,7 @@
       <c r="L74" s="2" t="n"/>
       <c r="M74" s="2" t="n"/>
     </row>
-    <row r="75" ht="20" customHeight="1">
+    <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -3651,7 +3651,7 @@
       <c r="L75" s="2" t="n"/>
       <c r="M75" s="2" t="n"/>
     </row>
-    <row r="76" ht="20" customHeight="1">
+    <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
           <t>Scopus</t>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Web Content</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -3785,7 +3785,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>iiitsurat.ac.in</t>
@@ -3826,7 +3826,7 @@
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>news.mit.edu</t>
@@ -3867,7 +3867,7 @@
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>www.getharvest.com</t>
@@ -4000,7 +4000,7 @@
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>www.ctm-it.com</t>
@@ -4065,12 +4065,12 @@
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>EC5</t>
-        </is>
-      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>IC1; IC2; IC4</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>YES</t>
@@ -4081,7 +4081,7 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>www.hse.ru</t>
@@ -4169,7 +4169,7 @@
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>www.thisdot.co</t>
@@ -4409,7 +4409,7 @@
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>towardsdatascience.com</t>
@@ -4450,7 +4450,7 @@
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>spb.hse.ru</t>
@@ -4603,7 +4603,7 @@
       <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>www.securityclearedjobs.com</t>
@@ -4644,7 +4644,7 @@
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>addyosmani.com</t>
@@ -4783,12 +4783,12 @@
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>IC1; IC3; IC5</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>EC5</t>
+        </is>
+      </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -4799,7 +4799,7 @@
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
     </row>
-    <row r="12" ht="20" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>careers.chevron.com</t>
@@ -4921,7 +4921,7 @@
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>society-rse.org</t>
@@ -4977,12 +4977,12 @@
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>EC3</t>
-        </is>
-      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>IC1</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
           <t>YES</t>
@@ -4993,7 +4993,7 @@
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>www.wearedevelopers.com</t>
@@ -5159,7 +5159,7 @@
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1">
+    <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>distantjob.com</t>

</xml_diff>